<commit_message>
Loop refresh: rescan + rebuild ledger
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0131Tm9QwYyPuHrkNkGr7Vys
</commit_message>
<xml_diff>
--- a/arb-scanner/data/Arbitrage_Ledger.xlsx
+++ b/arb-scanner/data/Arbitrage_Ledger.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-16 21:40 UTC from six live scanners: 11 crypto exchanges (~9,500 pairs), Polymarket + Kalshi order books,</t>
+          <t>Generated 2026-08-17 04:43 UTC from six live scanners: 11 crypto exchanges (~9,500 pairs), Polymarket + Kalshi order books,</t>
         </is>
       </c>
     </row>
@@ -936,87 +936,87 @@
         <v>1</v>
       </c>
       <c r="B4" s="10" t="n">
-        <v>5.48</v>
+        <v>5.17</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Locked carry</t>
+          <t>Rate arbitrage</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Delivery basis: WLD_USDT_20260821</t>
+          <t>Idle EUR: money-market ETF vs Greek deposit</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Gate futures</t>
+          <t>XEON/CSH2 via EU broker</t>
         </is>
       </c>
       <c r="F4" s="12" t="n">
-        <v>62.82</v>
+        <v>1.9</v>
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>% APR locked to expiry</t>
+          <t>% per year (2.19% ESTR - ~0.3% bank)</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>4.7d to delivery</t>
+          <t>one-time setup</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>weekly (new contracts)</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="J4" s="13" t="n">
-        <v>100000</v>
+        <v>10000000</v>
       </c>
       <c r="K4" s="11" t="inlineStr">
         <is>
-          <t>mark vs spot mid</t>
+          <t>ECB ESTR fix 2.188% (fetched)</t>
         </is>
       </c>
       <c r="L4" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M4" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="11" t="inlineStr">
+        <is>
+          <t>Near-riskless (o/n rates); ETF spread ~2bp; ESTR moves with ECB policy</t>
+        </is>
+      </c>
+      <c r="O4" s="11" t="inlineStr">
+        <is>
+          <t>Move idle EUR from Greek bank deposit to an overnight-rate MMF ETF</t>
+        </is>
+      </c>
+      <c r="P4" s="14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-17 04:43 UTC</t>
+        </is>
+      </c>
+      <c r="R4" s="15" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="S4" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="T4" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="U4" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="V4" s="15" t="n">
         <v>2</v>
-      </c>
-      <c r="N4" s="11" t="inlineStr">
-        <is>
-          <t>Margin on short leg; locked only if held to delivery</t>
-        </is>
-      </c>
-      <c r="O4" s="11" t="inlineStr">
-        <is>
-          <t>Buy spot + short dated future; converge at delivery regardless of price</t>
-        </is>
-      </c>
-      <c r="P4" s="14" t="n">
-        <v>17.2</v>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>2026-08-16T14:45:46Z</t>
-        </is>
-      </c>
-      <c r="R4" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="S4" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="T4" s="15" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="U4" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="V4" s="15" t="n">
-        <v>4</v>
       </c>
       <c r="W4" s="16">
         <f>$S$2*R4+$T$2*S4+$U$2*T4+$V$2*U4-$W$2*V4</f>
@@ -1028,87 +1028,87 @@
         <v>2</v>
       </c>
       <c r="B5" s="10" t="n">
-        <v>5.17</v>
+        <v>4.92</v>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Rate arbitrage</t>
+          <t>Delta-neutral carry</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Idle EUR: money-market ETF vs Greek deposit</t>
+          <t>Double-perp funding: ACE</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>XEON/CSH2 via EU broker</t>
+          <t>gate + bitget</t>
         </is>
       </c>
       <c r="F5" s="12" t="n">
-        <v>1.9</v>
+        <v>3.166</v>
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>% per year (2.19% ESTR - ~0.3% bank)</t>
+          <t>% per day while spread lasts</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>one-time setup</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>continuous (rate 8h/4h/1h)</t>
         </is>
       </c>
       <c r="J5" s="13" t="n">
-        <v>10000000</v>
+        <v>50000</v>
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>ECB ESTR fix 2.188% (fetched)</t>
+          <t>funding feeds both venues</t>
         </is>
       </c>
       <c r="L5" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M5" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N5" s="11" t="inlineStr">
         <is>
-          <t>Near-riskless (o/n rates); ETF spread ~2bp; ESTR moves with ECB policy</t>
+          <t>Rates converge in days; liquidation buffers both legs; 4 fees round trip</t>
         </is>
       </c>
       <c r="O5" s="11" t="inlineStr">
         <is>
-          <t>Move idle EUR from Greek bank deposit to an overnight-rate MMF ETF</t>
+          <t>Long ACE perp on gate, short on bitget - zero price exposure</t>
         </is>
       </c>
       <c r="P5" s="14" t="n">
-        <v>0.5</v>
+        <v>158.3</v>
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>2026-08-16 21:40 UTC</t>
+          <t>2026-08-17T04:43:00Z</t>
         </is>
       </c>
       <c r="R5" s="15" t="n">
-        <v>0.4</v>
+        <v>6.4</v>
       </c>
       <c r="S5" s="15" t="n">
         <v>9</v>
       </c>
       <c r="T5" s="15" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="U5" s="15" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="V5" s="15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="W5" s="16">
         <f>$S$2*R5+$T$2*S5+$U$2*T5+$V$2*U5-$W$2*V5</f>
@@ -1120,87 +1120,87 @@
         <v>3</v>
       </c>
       <c r="B6" s="10" t="n">
-        <v>4.82</v>
+        <v>4.59</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Locked carry</t>
+          <t>Delta-neutral carry</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Delivery basis: UNI_USDT_20260821</t>
+          <t>Double-perp funding: WAL</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Gate futures</t>
+          <t>gate + bitget</t>
         </is>
       </c>
       <c r="F6" s="12" t="n">
-        <v>39.02</v>
+        <v>1.033</v>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>% APR locked to expiry</t>
+          <t>% per day while spread lasts</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>4.7d to delivery</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>weekly (new contracts)</t>
+          <t>continuous (rate 8h/4h/1h)</t>
         </is>
       </c>
       <c r="J6" s="13" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>mark vs spot mid</t>
+          <t>funding feeds both venues</t>
         </is>
       </c>
       <c r="L6" s="9" t="n">
         <v>3</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N6" s="11" t="inlineStr">
         <is>
-          <t>Margin on short leg; locked only if held to delivery</t>
+          <t>Rates converge in days; liquidation buffers both legs; 4 fees round trip</t>
         </is>
       </c>
       <c r="O6" s="11" t="inlineStr">
         <is>
-          <t>Buy spot + short dated future; converge at delivery regardless of price</t>
+          <t>Long WAL perp on gate, short on bitget - zero price exposure</t>
         </is>
       </c>
       <c r="P6" s="14" t="n">
-        <v>10.7</v>
+        <v>51.6</v>
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>2026-08-16T14:45:46Z</t>
+          <t>2026-08-17T04:43:00Z</t>
         </is>
       </c>
       <c r="R6" s="15" t="n">
-        <v>7.8</v>
+        <v>5.3</v>
       </c>
       <c r="S6" s="15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="T6" s="15" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="U6" s="15" t="n">
         <v>6</v>
       </c>
       <c r="V6" s="15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W6" s="16">
         <f>$S$2*R6+$T$2*S6+$U$2*T6+$V$2*U6-$W$2*V6</f>
@@ -1212,87 +1212,87 @@
         <v>4</v>
       </c>
       <c r="B7" s="10" t="n">
-        <v>4.75</v>
+        <v>4.47</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Locked carry</t>
+          <t>Delta-neutral carry</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Delivery basis: AVAX_USDT_20260821</t>
+          <t>Double-perp funding: HOME</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Gate futures</t>
+          <t>gate + bitget</t>
         </is>
       </c>
       <c r="F7" s="12" t="n">
-        <v>38.21</v>
+        <v>0.714</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>% APR locked to expiry</t>
+          <t>% per day while spread lasts</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>4.7d to delivery</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>weekly (new contracts)</t>
+          <t>continuous (rate 8h/4h/1h)</t>
         </is>
       </c>
       <c r="J7" s="13" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>mark vs spot mid</t>
+          <t>funding feeds both venues</t>
         </is>
       </c>
       <c r="L7" s="9" t="n">
         <v>3</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N7" s="11" t="inlineStr">
         <is>
-          <t>Margin on short leg; locked only if held to delivery</t>
+          <t>Rates converge in days; liquidation buffers both legs; 4 fees round trip</t>
         </is>
       </c>
       <c r="O7" s="11" t="inlineStr">
         <is>
-          <t>Buy spot + short dated future; converge at delivery regardless of price</t>
+          <t>Long HOME perp on gate, short on bitget - zero price exposure</t>
         </is>
       </c>
       <c r="P7" s="14" t="n">
-        <v>10.5</v>
+        <v>35.7</v>
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>2026-08-16T14:45:46Z</t>
+          <t>2026-08-17T04:43:00Z</t>
         </is>
       </c>
       <c r="R7" s="15" t="n">
-        <v>7.6</v>
+        <v>4.9</v>
       </c>
       <c r="S7" s="15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="T7" s="15" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="U7" s="15" t="n">
         <v>6</v>
       </c>
       <c r="V7" s="15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W7" s="16">
         <f>$S$2*R7+$T$2*S7+$U$2*T7+$V$2*U7-$W$2*V7</f>
@@ -1304,87 +1304,87 @@
         <v>5</v>
       </c>
       <c r="B8" s="10" t="n">
-        <v>4.71</v>
+        <v>4.25</v>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Delta-neutral carry</t>
+          <t>Prediction structural</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Double-perp funding: ACE</t>
+          <t>Neg-risk sweep: Fed Decision in December?</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>gate + bitget</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="F8" s="12" t="n">
-        <v>1.521</v>
+        <v>0.251</v>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>% per day while spread lasts</t>
+          <t>% per cycle (riskless)</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>minutes</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>continuous (rate 8h/4h/1h)</t>
+          <t>5-20 (as books refill)</t>
         </is>
       </c>
       <c r="J8" s="13" t="n">
-        <v>50000</v>
+        <v>3120</v>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>funding feeds both venues</t>
+          <t>live CLOB, every outcome book</t>
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N8" s="11" t="inlineStr">
         <is>
-          <t>Rates converge in days; liquidation buffers both legs; 4 fees round trip</t>
+          <t>Depth-capped; edge locked at fill; no-fee venue</t>
         </is>
       </c>
       <c r="O8" s="11" t="inlineStr">
         <is>
-          <t>Long ACE perp on gate, short on bitget - zero price exposure</t>
+          <t>Buy NO on all 5 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P8" s="14" t="n">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>2026-08-16T14:45:46Z</t>
+          <t>2026-08-17T04:42:19Z</t>
         </is>
       </c>
       <c r="R8" s="15" t="n">
-        <v>5.7</v>
+        <v>2.9</v>
       </c>
       <c r="S8" s="15" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="T8" s="15" t="n">
-        <v>7</v>
+        <v>5.2</v>
       </c>
       <c r="U8" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V8" s="15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W8" s="16">
         <f>$S$2*R8+$T$2*S8+$U$2*T8+$V$2*U8-$W$2*V8</f>
@@ -1396,87 +1396,87 @@
         <v>6</v>
       </c>
       <c r="B9" s="10" t="n">
-        <v>4.68</v>
+        <v>4.12</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Delta-neutral carry</t>
+          <t>Prediction structural</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Double-perp funding: WAL</t>
+          <t>Neg-risk sweep: RC Celta de Vigo vs. CA Osasuna</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>gate + bitget</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.379</v>
+        <v>0.503</v>
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>% per day while spread lasts</t>
+          <t>% per cycle (riskless)</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>minutes</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>continuous (rate 8h/4h/1h)</t>
+          <t>5-20 (as books refill)</t>
         </is>
       </c>
       <c r="J9" s="13" t="n">
-        <v>50000</v>
+        <v>116</v>
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>funding feeds both venues</t>
+          <t>live CLOB, every outcome book</t>
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N9" s="11" t="inlineStr">
         <is>
-          <t>Rates converge in days; liquidation buffers both legs; 4 fees round trip</t>
+          <t>Depth-capped; edge locked at fill; no-fee venue</t>
         </is>
       </c>
       <c r="O9" s="11" t="inlineStr">
         <is>
-          <t>Long WAL perp on gate, short on bitget - zero price exposure</t>
+          <t>Buy NO on all 3 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P9" s="14" t="n">
-        <v>69</v>
+        <v>4.6</v>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>2026-08-16T14:45:46Z</t>
+          <t>2026-08-17T04:42:19Z</t>
         </is>
       </c>
       <c r="R9" s="15" t="n">
-        <v>5.6</v>
+        <v>3.5</v>
       </c>
       <c r="S9" s="15" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="T9" s="15" t="n">
-        <v>7</v>
+        <v>3.1</v>
       </c>
       <c r="U9" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V9" s="15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W9" s="16">
         <f>$S$2*R9+$T$2*S9+$U$2*T9+$V$2*U9-$W$2*V9</f>
@@ -1488,87 +1488,87 @@
         <v>7</v>
       </c>
       <c r="B10" s="10" t="n">
-        <v>4.65</v>
+        <v>4.02</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Delta-neutral carry</t>
+          <t>Prediction structural</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Double-perp funding: HOME</t>
+          <t>Neg-risk sweep: Fed Decision in October?</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>gate + bitget</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="F10" s="12" t="n">
-        <v>1.295</v>
+        <v>0.226</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>% per day while spread lasts</t>
+          <t>% per cycle (riskless)</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>minutes</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>continuous (rate 8h/4h/1h)</t>
+          <t>5-20 (as books refill)</t>
         </is>
       </c>
       <c r="J10" s="13" t="n">
-        <v>50000</v>
+        <v>399</v>
       </c>
       <c r="K10" s="11" t="inlineStr">
         <is>
-          <t>funding feeds both venues</t>
+          <t>live CLOB, every outcome book</t>
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N10" s="11" t="inlineStr">
         <is>
-          <t>Rates converge in days; liquidation buffers both legs; 4 fees round trip</t>
+          <t>Depth-capped; edge locked at fill; no-fee venue</t>
         </is>
       </c>
       <c r="O10" s="11" t="inlineStr">
         <is>
-          <t>Long HOME perp on gate, short on bitget - zero price exposure</t>
+          <t>Buy NO on all 5 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P10" s="14" t="n">
-        <v>64.8</v>
+        <v>7.2</v>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>2026-08-16T14:45:46Z</t>
+          <t>2026-08-17T04:42:19Z</t>
         </is>
       </c>
       <c r="R10" s="15" t="n">
-        <v>5.5</v>
+        <v>2.8</v>
       </c>
       <c r="S10" s="15" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="T10" s="15" t="n">
-        <v>7</v>
+        <v>3.9</v>
       </c>
       <c r="U10" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V10" s="15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W10" s="16">
         <f>$S$2*R10+$T$2*S10+$U$2*T10+$V$2*U10-$W$2*V10</f>
@@ -1580,7 +1580,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="10" t="n">
-        <v>4.46</v>
+        <v>3.93</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: Philadelphia Union vs. Inter Miami CF</t>
+          <t>Neg-risk sweep: Beşiktaş JK vs. FK Kauno Žalgiris</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -1598,7 +1598,7 @@
         </is>
       </c>
       <c r="F11" s="12" t="n">
-        <v>1.523</v>
+        <v>0.604</v>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
@@ -1616,7 +1616,7 @@
         </is>
       </c>
       <c r="J11" s="13" t="n">
-        <v>133</v>
+        <v>10</v>
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
@@ -1640,21 +1640,21 @@
         </is>
       </c>
       <c r="P11" s="14" t="n">
-        <v>16.2</v>
+        <v>0.5</v>
       </c>
       <c r="Q11" s="9" t="inlineStr">
         <is>
-          <t>2026-08-16T20:57:49Z</t>
+          <t>2026-08-17T04:42:19Z</t>
         </is>
       </c>
       <c r="R11" s="15" t="n">
-        <v>4.6</v>
+        <v>3.7</v>
       </c>
       <c r="S11" s="15" t="n">
         <v>6</v>
       </c>
       <c r="T11" s="15" t="n">
-        <v>3.2</v>
+        <v>1.5</v>
       </c>
       <c r="U11" s="15" t="n">
         <v>8</v>
@@ -1672,87 +1672,87 @@
         <v>9</v>
       </c>
       <c r="B12" s="18" t="n">
-        <v>4.33</v>
+        <v>3.93</v>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>Prediction structural</t>
+          <t>DeFi rate arbitrage</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: RC Celta de Vigo vs. CA Osasuna</t>
+          <t>Borrow-lend spread: WETH on Base</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>compound-v3 -&gt; fusion-by-ipor</t>
         </is>
       </c>
       <c r="F12" s="20" t="n">
-        <v>1.01</v>
+        <v>8.1</v>
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>% per cycle (riskless)</t>
+          <t>% per year on borrowed notional</t>
         </is>
       </c>
       <c r="H12" s="19" t="inlineStr">
         <is>
-          <t>minutes</t>
+          <t>instant entry/exit</t>
         </is>
       </c>
       <c r="I12" s="19" t="inlineStr">
         <is>
-          <t>5-20 (as books refill)</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="J12" s="21" t="n">
-        <v>125</v>
+        <v>5115081</v>
       </c>
       <c r="K12" s="19" t="inlineStr">
         <is>
-          <t>live CLOB, every outcome book</t>
+          <t>DefiLlama live rates</t>
         </is>
       </c>
       <c r="L12" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M12" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Depth-capped; edge locked at fill; no-fee venue</t>
+          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
         </is>
       </c>
       <c r="O12" s="19" t="inlineStr">
         <is>
-          <t>Buy NO on all 3 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
+          <t>Borrow WETH at 0% on compound-v3, lend at 8.1% on fusion-by-ipor</t>
         </is>
       </c>
       <c r="P12" s="22" t="n">
-        <v>10.1</v>
+        <v>1.6</v>
       </c>
       <c r="Q12" s="17" t="inlineStr">
         <is>
-          <t>2026-08-16T20:57:49Z</t>
+          <t>2026-08-16T20:29:43Z</t>
         </is>
       </c>
       <c r="R12" s="15" t="n">
-        <v>4.2</v>
+        <v>1.6</v>
       </c>
       <c r="S12" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="T12" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="U12" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="T12" s="15" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="U12" s="15" t="n">
-        <v>8</v>
-      </c>
       <c r="V12" s="15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="W12" s="16">
         <f>$S$2*R12+$T$2*S12+$U$2*T12+$V$2*U12-$W$2*V12</f>
@@ -1764,87 +1764,87 @@
         <v>10</v>
       </c>
       <c r="B13" s="18" t="n">
-        <v>3.95</v>
+        <v>3.9</v>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>Prediction structural</t>
+          <t>Rate arbitrage</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: GPU rental prices (H100) end of August?</t>
+          <t>EURC on-chain vs Greek deposit</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Aave v3 Ethereum</t>
         </is>
       </c>
       <c r="F13" s="20" t="n">
-        <v>0.261</v>
+        <v>2.6</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>% per cycle (riskless)</t>
+          <t>% per year net of bank rate</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>minutes</t>
+          <t>instant</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>5-20 (as books refill)</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="J13" s="21" t="n">
-        <v>130</v>
+        <v>11000000</v>
       </c>
       <c r="K13" s="19" t="inlineStr">
         <is>
-          <t>live CLOB, every outcome book</t>
+          <t>DefiLlama: EURC 2.93% APY, $11M TVL</t>
         </is>
       </c>
       <c r="L13" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="M13" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" s="19" t="inlineStr">
+        <is>
+          <t>Smart-contract + stablecoin issuer risk; beats ESTR slightly</t>
+        </is>
+      </c>
+      <c r="O13" s="19" t="inlineStr">
+        <is>
+          <t>Hold EURC, supply on Aave</t>
+        </is>
+      </c>
+      <c r="P13" s="22" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Q13" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-17 04:43 UTC</t>
+        </is>
+      </c>
+      <c r="R13" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S13" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="T13" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="U13" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="V13" s="15" t="n">
         <v>4</v>
-      </c>
-      <c r="M13" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" s="19" t="inlineStr">
-        <is>
-          <t>Depth-capped; edge locked at fill; no-fee venue</t>
-        </is>
-      </c>
-      <c r="O13" s="19" t="inlineStr">
-        <is>
-          <t>Buy NO on all 6 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
-        </is>
-      </c>
-      <c r="P13" s="22" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="Q13" s="17" t="inlineStr">
-        <is>
-          <t>2026-08-16T20:57:49Z</t>
-        </is>
-      </c>
-      <c r="R13" s="15" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="S13" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="T13" s="15" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="U13" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="V13" s="15" t="n">
-        <v>2</v>
       </c>
       <c r="W13" s="16">
         <f>$S$2*R13+$T$2*S13+$U$2*T13+$V$2*U13-$W$2*V13</f>
@@ -1856,67 +1856,67 @@
         <v>11</v>
       </c>
       <c r="B14" s="18" t="n">
-        <v>3.93</v>
+        <v>3.87</v>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>DeFi rate arbitrage</t>
+          <t>Gaming items</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Borrow-lend spread: WETH on Base</t>
+          <t>CS2 skins spend-discount (median 22.1% off Steam)</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
-          <t>compound-v3 -&gt; fusion-by-ipor</t>
+          <t>Skinport -&gt; Steam ecosystem</t>
         </is>
       </c>
       <c r="F14" s="20" t="n">
-        <v>8.1</v>
+        <v>22.1</v>
       </c>
       <c r="G14" s="19" t="inlineStr">
         <is>
-          <t>% per year on borrowed notional</t>
+          <t>% discount on Steam spend</t>
         </is>
       </c>
       <c r="H14" s="19" t="inlineStr">
         <is>
-          <t>instant entry/exit</t>
+          <t>instant</t>
         </is>
       </c>
       <c r="I14" s="19" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>unlimited for own spending</t>
         </is>
       </c>
       <c r="J14" s="21" t="n">
-        <v>5115081</v>
+        <v>1000</v>
       </c>
       <c r="K14" s="19" t="inlineStr">
         <is>
-          <t>DefiLlama live rates</t>
+          <t>full 21k-item catalog</t>
         </is>
       </c>
       <c r="L14" s="17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M14" s="17" t="n">
         <v>3</v>
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
+          <t>ONE-WAY: Steam wallet cannot cash out - only worth it for money you'd spend on Steam anyway</t>
         </is>
       </c>
       <c r="O14" s="19" t="inlineStr">
         <is>
-          <t>Borrow WETH at 0% on compound-v3, lend at 8.1% on fusion-by-ipor</t>
+          <t>Buy discounted items on Skinport instead of paying Steam prices</t>
         </is>
       </c>
       <c r="P14" s="22" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="17" t="inlineStr">
         <is>
@@ -1924,16 +1924,16 @@
         </is>
       </c>
       <c r="R14" s="15" t="n">
-        <v>1.6</v>
+        <v>5.5</v>
       </c>
       <c r="S14" s="15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="T14" s="15" t="n">
-        <v>10</v>
+        <v>4.5</v>
       </c>
       <c r="U14" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V14" s="15" t="n">
         <v>6</v>
@@ -1948,7 +1948,7 @@
         <v>12</v>
       </c>
       <c r="B15" s="18" t="n">
-        <v>3.91</v>
+        <v>3.82</v>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
@@ -1957,7 +1957,7 @@
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: GPU rental prices (H200) end of August?</t>
+          <t>Ladder violation: Will Solana reach $320 by December 31, 2</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
@@ -1966,29 +1966,29 @@
         </is>
       </c>
       <c r="F15" s="20" t="n">
-        <v>0.2</v>
+        <v>1.11</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>% per cycle (riskless)</t>
+          <t>% locked at fill</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>minutes</t>
+          <t>instant fill; pays at resolution</t>
         </is>
       </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
-          <t>5-20 (as books refill)</t>
+          <t>when flagged (few/week)</t>
         </is>
       </c>
       <c r="J15" s="21" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>live CLOB, every outcome book</t>
+          <t>live CLOB depth</t>
         </is>
       </c>
       <c r="L15" s="17" t="n">
@@ -1999,30 +1999,30 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Depth-capped; edge locked at fill; no-fee venue</t>
+          <t>Riskless at fill; capital returns at event resolution; ~$50 size</t>
         </is>
       </c>
       <c r="O15" s="19" t="inlineStr">
         <is>
-          <t>Buy NO on all 6 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
+          <t>Buy YES weaker strike + NO stronger strike for &lt; $1/set; min payout $1, $2 if between strikes</t>
         </is>
       </c>
       <c r="P15" s="22" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="Q15" s="17" t="inlineStr">
         <is>
-          <t>2026-08-16T20:57:49Z</t>
+          <t>2026-08-17T04:43:00Z</t>
         </is>
       </c>
       <c r="R15" s="15" t="n">
-        <v>2.7</v>
+        <v>4.3</v>
       </c>
       <c r="S15" s="15" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T15" s="15" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
       <c r="U15" s="15" t="n">
         <v>8</v>
@@ -2040,34 +2040,34 @@
         <v>13</v>
       </c>
       <c r="B16" s="18" t="n">
-        <v>3.9</v>
+        <v>3.82</v>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>Rate arbitrage</t>
+          <t>DeFi rate arbitrage</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>EURC on-chain vs Greek deposit</t>
+          <t>Borrow-lend spread: USD3 on Ethereum</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>Aave v3 Ethereum</t>
+          <t>morpho-blue -&gt; pendle</t>
         </is>
       </c>
       <c r="F16" s="20" t="n">
-        <v>2.6</v>
+        <v>7.12</v>
       </c>
       <c r="G16" s="19" t="inlineStr">
         <is>
-          <t>% per year net of bank rate</t>
+          <t>% per year on borrowed notional</t>
         </is>
       </c>
       <c r="H16" s="19" t="inlineStr">
         <is>
-          <t>instant</t>
+          <t>instant entry/exit</t>
         </is>
       </c>
       <c r="I16" s="19" t="inlineStr">
@@ -2076,51 +2076,51 @@
         </is>
       </c>
       <c r="J16" s="21" t="n">
-        <v>11000000</v>
+        <v>2763264</v>
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>DefiLlama: EURC 2.93% APY, $11M TVL</t>
+          <t>DefiLlama live rates</t>
         </is>
       </c>
       <c r="L16" s="17" t="n">
         <v>3</v>
       </c>
       <c r="M16" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Smart-contract + stablecoin issuer risk; beats ESTR slightly</t>
+          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
         </is>
       </c>
       <c r="O16" s="19" t="inlineStr">
         <is>
-          <t>Hold EURC, supply on Aave</t>
+          <t>Borrow USD3 at 7.27% on morpho-blue, lend at 14.39% on pendle</t>
         </is>
       </c>
       <c r="P16" s="22" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="Q16" s="17" t="inlineStr">
         <is>
-          <t>2026-08-16 21:40 UTC</t>
+          <t>2026-08-16T20:29:43Z</t>
         </is>
       </c>
       <c r="R16" s="15" t="n">
-        <v>0.5</v>
+        <v>1.4</v>
       </c>
       <c r="S16" s="15" t="n">
         <v>9</v>
       </c>
       <c r="T16" s="15" t="n">
-        <v>10</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="U16" s="15" t="n">
         <v>6</v>
       </c>
       <c r="V16" s="15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W16" s="16">
         <f>$S$2*R16+$T$2*S16+$U$2*T16+$V$2*U16-$W$2*V16</f>
@@ -2132,67 +2132,67 @@
         <v>14</v>
       </c>
       <c r="B17" s="18" t="n">
-        <v>3.87</v>
+        <v>3.81</v>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>Gaming items</t>
+          <t>DeFi rate arbitrage</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>CS2 skins spend-discount (median 22.1% off Steam)</t>
+          <t>Borrow-lend spread: USDC on Solana</t>
         </is>
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>Skinport -&gt; Steam ecosystem</t>
+          <t>kamino-lend -&gt; neutral-trade</t>
         </is>
       </c>
       <c r="F17" s="20" t="n">
-        <v>22.1</v>
+        <v>8.31</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>% discount on Steam spend</t>
+          <t>% per year on borrowed notional</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>instant</t>
+          <t>instant entry/exit</t>
         </is>
       </c>
       <c r="I17" s="19" t="inlineStr">
         <is>
-          <t>unlimited for own spending</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="J17" s="21" t="n">
-        <v>1000</v>
+        <v>1066804</v>
       </c>
       <c r="K17" s="19" t="inlineStr">
         <is>
-          <t>full 21k-item catalog</t>
+          <t>DefiLlama live rates</t>
         </is>
       </c>
       <c r="L17" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M17" s="17" t="n">
         <v>3</v>
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>ONE-WAY: Steam wallet cannot cash out - only worth it for money you'd spend on Steam anyway</t>
+          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
         </is>
       </c>
       <c r="O17" s="19" t="inlineStr">
         <is>
-          <t>Buy discounted items on Skinport instead of paying Steam prices</t>
+          <t>Borrow USDC at 2.57% on kamino-lend, lend at 10.89% on neutral-trade</t>
         </is>
       </c>
       <c r="P17" s="22" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="Q17" s="17" t="inlineStr">
         <is>
@@ -2200,16 +2200,16 @@
         </is>
       </c>
       <c r="R17" s="15" t="n">
-        <v>5.5</v>
+        <v>1.7</v>
       </c>
       <c r="S17" s="15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="T17" s="15" t="n">
-        <v>4.5</v>
+        <v>9</v>
       </c>
       <c r="U17" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V17" s="15" t="n">
         <v>6</v>
@@ -2224,7 +2224,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="18" t="n">
-        <v>3.86</v>
+        <v>3.8</v>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: Anthropic IPO Closing Market Cap</t>
+          <t>Neg-risk sweep: Highest temperature in Buenos Aires on August</t>
         </is>
       </c>
       <c r="E18" s="17" t="inlineStr">
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="F18" s="20" t="n">
-        <v>0.245</v>
+        <v>0.241</v>
       </c>
       <c r="G18" s="19" t="inlineStr">
         <is>
@@ -2260,7 +2260,7 @@
         </is>
       </c>
       <c r="J18" s="21" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="K18" s="19" t="inlineStr">
         <is>
@@ -2280,25 +2280,25 @@
       </c>
       <c r="O18" s="19" t="inlineStr">
         <is>
-          <t>Buy NO on all 10 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
+          <t>Buy NO on all 11 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P18" s="22" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="Q18" s="17" t="inlineStr">
         <is>
-          <t>2026-08-16T20:57:49Z</t>
+          <t>2026-08-17T04:42:19Z</t>
         </is>
       </c>
       <c r="R18" s="15" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="S18" s="15" t="n">
         <v>6</v>
       </c>
       <c r="T18" s="15" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="U18" s="15" t="n">
         <v>8</v>
@@ -2316,7 +2316,7 @@
         <v>16</v>
       </c>
       <c r="B19" s="18" t="n">
-        <v>3.83</v>
+        <v>3.79</v>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: James Fishback vote share in 2026 Florida Rep</t>
+          <t>Neg-risk sweep: Al Ta'ee Saudi Club vs. Al Qadisiyah Saudi Cl</t>
         </is>
       </c>
       <c r="E19" s="17" t="inlineStr">
@@ -2334,7 +2334,7 @@
         </is>
       </c>
       <c r="F19" s="20" t="n">
-        <v>0.18</v>
+        <v>0.351</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
@@ -2352,7 +2352,7 @@
         </is>
       </c>
       <c r="J19" s="21" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="K19" s="19" t="inlineStr">
         <is>
@@ -2372,25 +2372,25 @@
       </c>
       <c r="O19" s="19" t="inlineStr">
         <is>
-          <t>Buy NO on all 6 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
+          <t>Buy NO on all 3 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P19" s="22" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="17" t="inlineStr">
         <is>
-          <t>2026-08-16T20:57:49Z</t>
+          <t>2026-08-17T04:42:19Z</t>
         </is>
       </c>
       <c r="R19" s="15" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="S19" s="15" t="n">
         <v>6</v>
       </c>
       <c r="T19" s="15" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="U19" s="15" t="n">
         <v>8</v>
@@ -2408,87 +2408,87 @@
         <v>17</v>
       </c>
       <c r="B20" s="23" t="n">
-        <v>3.82</v>
+        <v>3.78</v>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>Prediction structural</t>
+          <t>P2P fiat corridor</t>
         </is>
       </c>
       <c r="D20" s="24" t="inlineStr">
         <is>
-          <t>Ladder violation: Will Solana reach $320 by December 31, 2</t>
+          <t>EUR clean same-platform loop</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>OKX P2P (Dukascopy legs)</t>
         </is>
       </c>
       <c r="F20" s="16" t="n">
-        <v>1.11</v>
+        <v>0.34</v>
       </c>
       <c r="G20" s="24" t="inlineStr">
         <is>
-          <t>% locked at fill</t>
+          <t>% per cycle</t>
         </is>
       </c>
       <c r="H20" s="24" t="inlineStr">
         <is>
-          <t>instant fill; pays at resolution</t>
+          <t>10-30 min per leg</t>
         </is>
       </c>
       <c r="I20" s="24" t="inlineStr">
         <is>
-          <t>when flagged (few/week)</t>
+          <t>5-15</t>
         </is>
       </c>
       <c r="J20" s="25" t="n">
-        <v>50</v>
+        <v>5000</v>
       </c>
       <c r="K20" s="24" t="inlineStr">
         <is>
-          <t>live CLOB depth</t>
+          <t>live books</t>
         </is>
       </c>
       <c r="L20" s="15" t="n">
         <v>4</v>
       </c>
       <c r="M20" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N20" s="24" t="inlineStr">
         <is>
-          <t>Riskless at fill; capital returns at event resolution; ~$50 size</t>
+          <t>Thin EUR books; above-fair offers are fraud bait (mule risk) - trade only at fair prices</t>
         </is>
       </c>
       <c r="O20" s="24" t="inlineStr">
         <is>
-          <t>Buy YES weaker strike + NO stronger strike for &lt; $1/set; min payout $1, $2 if between strikes</t>
+          <t>Buy/sell USDT vs EUR on same payment platform at the clean spread</t>
         </is>
       </c>
       <c r="P20" s="26" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q20" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16T14:45:46Z</t>
+          <t>2026-08-16T20:29:43Z</t>
         </is>
       </c>
       <c r="R20" s="15" t="n">
-        <v>4.3</v>
+        <v>3.2</v>
       </c>
       <c r="S20" s="15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T20" s="15" t="n">
-        <v>2.5</v>
+        <v>5.5</v>
       </c>
       <c r="U20" s="15" t="n">
         <v>8</v>
       </c>
       <c r="V20" s="15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="W20" s="16">
         <f>$S$2*R20+$T$2*S20+$U$2*T20+$V$2*U20-$W$2*V20</f>
@@ -2500,87 +2500,87 @@
         <v>18</v>
       </c>
       <c r="B21" s="23" t="n">
-        <v>3.82</v>
+        <v>3.75</v>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>DeFi rate arbitrage</t>
+          <t>Prediction structural</t>
         </is>
       </c>
       <c r="D21" s="24" t="inlineStr">
         <is>
-          <t>Borrow-lend spread: USD3 on Ethereum</t>
+          <t>Ladder violation: Will Solana reach $300 by December 31, 2</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>morpho-blue -&gt; pendle</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="F21" s="16" t="n">
-        <v>7.12</v>
+        <v>0.91</v>
       </c>
       <c r="G21" s="24" t="inlineStr">
         <is>
-          <t>% per year on borrowed notional</t>
+          <t>% locked at fill</t>
         </is>
       </c>
       <c r="H21" s="24" t="inlineStr">
         <is>
-          <t>instant entry/exit</t>
+          <t>instant fill; pays at resolution</t>
         </is>
       </c>
       <c r="I21" s="24" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>when flagged (few/week)</t>
         </is>
       </c>
       <c r="J21" s="25" t="n">
-        <v>2763264</v>
+        <v>50</v>
       </c>
       <c r="K21" s="24" t="inlineStr">
         <is>
-          <t>DefiLlama live rates</t>
+          <t>live CLOB depth</t>
         </is>
       </c>
       <c r="L21" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="M21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" s="24" t="inlineStr">
+        <is>
+          <t>Riskless at fill; capital returns at event resolution; ~$50 size</t>
+        </is>
+      </c>
+      <c r="O21" s="24" t="inlineStr">
+        <is>
+          <t>Buy YES weaker strike + NO stronger strike for &lt; $1/set; min payout $1, $2 if between strikes</t>
+        </is>
+      </c>
+      <c r="P21" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q21" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-17T04:43:00Z</t>
+        </is>
+      </c>
+      <c r="R21" s="15" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="S21" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="M21" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="N21" s="24" t="inlineStr">
-        <is>
-          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
-        </is>
-      </c>
-      <c r="O21" s="24" t="inlineStr">
-        <is>
-          <t>Borrow USD3 at 7.27% on morpho-blue, lend at 14.39% on pendle</t>
-        </is>
-      </c>
-      <c r="P21" s="26" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="Q21" s="15" t="inlineStr">
-        <is>
-          <t>2026-08-16T20:29:43Z</t>
-        </is>
-      </c>
-      <c r="R21" s="15" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="S21" s="15" t="n">
-        <v>9</v>
-      </c>
       <c r="T21" s="15" t="n">
-        <v>9.699999999999999</v>
+        <v>2.5</v>
       </c>
       <c r="U21" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V21" s="15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W21" s="16">
         <f>$S$2*R21+$T$2*S21+$U$2*T21+$V$2*U21-$W$2*V21</f>
@@ -2592,87 +2592,87 @@
         <v>19</v>
       </c>
       <c r="B22" s="23" t="n">
-        <v>3.81</v>
+        <v>3.63</v>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>DeFi rate arbitrage</t>
+          <t>Market-making</t>
         </is>
       </c>
       <c r="D22" s="24" t="inlineStr">
         <is>
-          <t>Borrow-lend spread: USDC on Solana</t>
+          <t>Spread capture: RAZORUSDT (mexc)</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>kamino-lend -&gt; neutral-trade</t>
+          <t>mexc</t>
         </is>
       </c>
       <c r="F22" s="16" t="n">
-        <v>8.31</v>
+        <v>2.6549</v>
       </c>
       <c r="G22" s="24" t="inlineStr">
         <is>
-          <t>% per year on borrowed notional</t>
+          <t>% per round trip</t>
         </is>
       </c>
       <c r="H22" s="24" t="inlineStr">
         <is>
-          <t>instant entry/exit</t>
+          <t>minutes per RT</t>
         </is>
       </c>
       <c r="I22" s="24" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>10-100 fills</t>
         </is>
       </c>
       <c r="J22" s="25" t="n">
-        <v>1066804</v>
+        <v>500</v>
       </c>
       <c r="K22" s="24" t="inlineStr">
         <is>
-          <t>DefiLlama live rates</t>
+          <t>live books + trade tape</t>
         </is>
       </c>
       <c r="L22" s="15" t="n">
         <v>3</v>
       </c>
       <c r="M22" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N22" s="24" t="inlineStr">
         <is>
-          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
+          <t>INVENTORY RISK: one-sided fills accumulate positions; microcaps gap hard; sim showed +/-$90 swings vs $8 capture</t>
         </is>
       </c>
       <c r="O22" s="24" t="inlineStr">
         <is>
-          <t>Borrow USDC at 2.57% on kamino-lend, lend at 10.89% on neutral-trade</t>
+          <t>Post maker bid+ask inside the spread (0% maker on MEXC); manage inventory</t>
         </is>
       </c>
       <c r="P22" s="26" t="n">
-        <v>1.6</v>
+        <v>15</v>
       </c>
       <c r="Q22" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16T20:29:43Z</t>
+          <t>2026-08-17 04:43 UTC</t>
         </is>
       </c>
       <c r="R22" s="15" t="n">
-        <v>1.7</v>
+        <v>5.1</v>
       </c>
       <c r="S22" s="15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T22" s="15" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="U22" s="15" t="n">
         <v>6</v>
       </c>
       <c r="V22" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="W22" s="16">
         <f>$S$2*R22+$T$2*S22+$U$2*T22+$V$2*U22-$W$2*V22</f>
@@ -2684,87 +2684,87 @@
         <v>20</v>
       </c>
       <c r="B23" s="23" t="n">
-        <v>3.78</v>
+        <v>3.63</v>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>P2P fiat corridor</t>
+          <t>Market-making</t>
         </is>
       </c>
       <c r="D23" s="24" t="inlineStr">
         <is>
-          <t>EUR clean same-platform loop</t>
+          <t>In-play sports MM (nightly games)</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>OKX P2P (Dukascopy legs)</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="F23" s="16" t="n">
-        <v>0.34</v>
+        <v>1.5</v>
       </c>
       <c r="G23" s="24" t="inlineStr">
         <is>
-          <t>% per cycle</t>
+          <t>% of mid per round trip</t>
         </is>
       </c>
       <c r="H23" s="24" t="inlineStr">
         <is>
-          <t>10-30 min per leg</t>
+          <t>seconds-minutes per RT</t>
         </is>
       </c>
       <c r="I23" s="24" t="inlineStr">
         <is>
-          <t>5-15</t>
+          <t>100s during games</t>
         </is>
       </c>
       <c r="J23" s="25" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="K23" s="24" t="inlineStr">
         <is>
-          <t>live books</t>
+          <t>CLOB depth + trade tape</t>
         </is>
       </c>
       <c r="L23" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M23" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="M23" s="15" t="n">
-        <v>3</v>
-      </c>
       <c r="N23" s="24" t="inlineStr">
         <is>
-          <t>Thin EUR books; above-fair offers are fraud bait (mule risk) - trade only at fair prices</t>
+          <t>Adverse selection on goals/rounds; must pull quotes near resolution; no fees</t>
         </is>
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>Buy/sell USDT vs EUR on same payment platform at the clean spread</t>
+          <t>Quote both sides of live game books (1-4c spreads, 1000s prints/hr); fresh books daily</t>
         </is>
       </c>
       <c r="P23" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q23" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-17 04:43 UTC</t>
+        </is>
+      </c>
+      <c r="R23" s="15" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="S23" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="T23" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="Q23" s="15" t="inlineStr">
-        <is>
-          <t>2026-08-16T20:29:43Z</t>
-        </is>
-      </c>
-      <c r="R23" s="15" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="S23" s="15" t="n">
+      <c r="U23" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="T23" s="15" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="U23" s="15" t="n">
+      <c r="V23" s="15" t="n">
         <v>8</v>
-      </c>
-      <c r="V23" s="15" t="n">
-        <v>6</v>
       </c>
       <c r="W23" s="16">
         <f>$S$2*R23+$T$2*S23+$U$2*T23+$V$2*U23-$W$2*V23</f>
@@ -2776,87 +2776,87 @@
         <v>21</v>
       </c>
       <c r="B24" s="23" t="n">
-        <v>3.75</v>
+        <v>3.6</v>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>Prediction structural</t>
+          <t>Market-making</t>
         </is>
       </c>
       <c r="D24" s="24" t="inlineStr">
         <is>
-          <t>Ladder violation: Will Solana reach $300 by December 31, 2</t>
+          <t>Spread capture: MAPO-USDT (kucoin)</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>kucoin</t>
         </is>
       </c>
       <c r="F24" s="16" t="n">
-        <v>0.91</v>
+        <v>2.234</v>
       </c>
       <c r="G24" s="24" t="inlineStr">
         <is>
-          <t>% locked at fill</t>
+          <t>% per round trip</t>
         </is>
       </c>
       <c r="H24" s="24" t="inlineStr">
         <is>
-          <t>instant fill; pays at resolution</t>
+          <t>minutes per RT</t>
         </is>
       </c>
       <c r="I24" s="24" t="inlineStr">
         <is>
-          <t>when flagged (few/week)</t>
+          <t>10-100 fills</t>
         </is>
       </c>
       <c r="J24" s="25" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="K24" s="24" t="inlineStr">
         <is>
-          <t>live CLOB depth</t>
+          <t>live books + trade tape</t>
         </is>
       </c>
       <c r="L24" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M24" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="M24" s="15" t="n">
-        <v>1</v>
-      </c>
       <c r="N24" s="24" t="inlineStr">
         <is>
-          <t>Riskless at fill; capital returns at event resolution; ~$50 size</t>
+          <t>INVENTORY RISK: one-sided fills accumulate positions; microcaps gap hard; sim showed +/-$90 swings vs $8 capture</t>
         </is>
       </c>
       <c r="O24" s="24" t="inlineStr">
         <is>
-          <t>Buy YES weaker strike + NO stronger strike for &lt; $1/set; min payout $1, $2 if between strikes</t>
+          <t>Post maker bid+ask inside the spread (0% maker on MEXC); manage inventory</t>
         </is>
       </c>
       <c r="P24" s="26" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="Q24" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16T14:45:46Z</t>
+          <t>2026-08-17 04:43 UTC</t>
         </is>
       </c>
       <c r="R24" s="15" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="S24" s="15" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="T24" s="15" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="U24" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="V24" s="15" t="n">
         <v>8</v>
-      </c>
-      <c r="V24" s="15" t="n">
-        <v>2</v>
       </c>
       <c r="W24" s="16">
         <f>$S$2*R24+$T$2*S24+$U$2*T24+$V$2*U24-$W$2*V24</f>
@@ -2868,7 +2868,7 @@
         <v>22</v>
       </c>
       <c r="B25" s="23" t="n">
-        <v>3.63</v>
+        <v>3.54</v>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="D25" s="24" t="inlineStr">
         <is>
-          <t>Spread capture: RAZORUSDT (mexc)</t>
+          <t>Spread capture: XPLKUSDT (mexc)</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
@@ -2886,7 +2886,7 @@
         </is>
       </c>
       <c r="F25" s="16" t="n">
-        <v>2.6549</v>
+        <v>1.9691</v>
       </c>
       <c r="G25" s="24" t="inlineStr">
         <is>
@@ -2932,11 +2932,11 @@
       </c>
       <c r="Q25" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16 21:40 UTC</t>
+          <t>2026-08-17 04:43 UTC</t>
         </is>
       </c>
       <c r="R25" s="15" t="n">
-        <v>5.1</v>
+        <v>4.8</v>
       </c>
       <c r="S25" s="15" t="n">
         <v>8</v>
@@ -2960,87 +2960,87 @@
         <v>23</v>
       </c>
       <c r="B26" s="23" t="n">
-        <v>3.63</v>
+        <v>3.51</v>
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>Market-making</t>
+          <t>Fixed-rate lock</t>
         </is>
       </c>
       <c r="D26" s="24" t="inlineStr">
         <is>
-          <t>In-play sports MM (nightly games)</t>
+          <t>Pendle PT stable yields (best liquid: 14-18% APY)</t>
         </is>
       </c>
       <c r="E26" s="15" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Pendle (Ethereum)</t>
         </is>
       </c>
       <c r="F26" s="16" t="n">
-        <v>1.5</v>
+        <v>16</v>
       </c>
       <c r="G26" s="24" t="inlineStr">
         <is>
-          <t>% of mid per round trip</t>
+          <t>% APY fixed at purchase</t>
         </is>
       </c>
       <c r="H26" s="24" t="inlineStr">
         <is>
-          <t>seconds-minutes per RT</t>
+          <t>instant buy; hold to maturity</t>
         </is>
       </c>
       <c r="I26" s="24" t="inlineStr">
         <is>
-          <t>100s during games</t>
+          <t>monthly (new maturities)</t>
         </is>
       </c>
       <c r="J26" s="25" t="n">
-        <v>2000</v>
+        <v>5000000</v>
       </c>
       <c r="K26" s="24" t="inlineStr">
         <is>
-          <t>CLOB depth + trade tape</t>
+          <t>Pendle API implied APY</t>
         </is>
       </c>
       <c r="L26" s="15" t="n">
         <v>3</v>
       </c>
       <c r="M26" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N26" s="24" t="inlineStr">
         <is>
-          <t>Adverse selection on goals/rounds; must pull quotes near resolution; no fees</t>
+          <t>Underlying protocol/stablecoin solvency is the paid risk; yield locked only to maturity</t>
         </is>
       </c>
       <c r="O26" s="24" t="inlineStr">
         <is>
-          <t>Quote both sides of live game books (1-4c spreads, 1000s prints/hr); fresh books daily</t>
+          <t>Buy discounted principal token, redeem at par at maturity</t>
         </is>
       </c>
       <c r="P26" s="26" t="n">
-        <v>25</v>
+        <v>4.4</v>
       </c>
       <c r="Q26" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16 21:40 UTC</t>
+          <t>2026-08-17 04:43 UTC</t>
         </is>
       </c>
       <c r="R26" s="15" t="n">
-        <v>4.6</v>
+        <v>3.2</v>
       </c>
       <c r="S26" s="15" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="T26" s="15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="U26" s="15" t="n">
         <v>6</v>
       </c>
       <c r="V26" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W26" s="16">
         <f>$S$2*R26+$T$2*S26+$U$2*T26+$V$2*U26-$W$2*V26</f>
@@ -3052,87 +3052,87 @@
         <v>24</v>
       </c>
       <c r="B27" s="23" t="n">
-        <v>3.6</v>
+        <v>3.04</v>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>Market-making</t>
+          <t>P2P fiat corridor</t>
         </is>
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>Spread capture: MAPO-USDT (kucoin)</t>
+          <t>Ukraine in-country loop (PrivatBank both legs)</t>
         </is>
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>kucoin</t>
+          <t>OKX P2P</t>
         </is>
       </c>
       <c r="F27" s="16" t="n">
-        <v>2.234</v>
+        <v>2.8</v>
       </c>
       <c r="G27" s="24" t="inlineStr">
         <is>
-          <t>% per round trip</t>
+          <t>% per cycle</t>
         </is>
       </c>
       <c r="H27" s="24" t="inlineStr">
         <is>
-          <t>minutes per RT</t>
+          <t>5-15 min per leg</t>
         </is>
       </c>
       <c r="I27" s="24" t="inlineStr">
         <is>
-          <t>10-100 fills</t>
+          <t>20-40</t>
         </is>
       </c>
       <c r="J27" s="25" t="n">
-        <v>500</v>
+        <v>20000</v>
       </c>
       <c r="K27" s="24" t="inlineStr">
         <is>
-          <t>live books + trade tape</t>
-        </is>
-      </c>
-      <c r="L27" s="15" t="n">
+          <t>offer-level check incl. depth+banks</t>
+        </is>
+      </c>
+      <c r="L27" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="M27" s="15" t="n">
-        <v>4</v>
-      </c>
       <c r="N27" s="24" t="inlineStr">
         <is>
-          <t>INVENTORY RISK: one-sided fills accumulate positions; microcaps gap hard; sim showed +/-$90 swings vs $8 capture</t>
+          <t>REQUIRES Ukrainian bank rails - not executable from Greece; counterparty/chargeback risk</t>
         </is>
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>Post maker bid+ask inside the spread (0% maker on MEXC); manage inventory</t>
+          <t>Buy USDT from merchant A, sell to merchant B, same bank transfers</t>
         </is>
       </c>
       <c r="P27" s="26" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="Q27" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16 21:40 UTC</t>
+          <t>2026-08-16T20:29:43Z</t>
         </is>
       </c>
       <c r="R27" s="15" t="n">
-        <v>5</v>
+        <v>5.2</v>
       </c>
       <c r="S27" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="T27" s="15" t="n">
-        <v>4</v>
+        <v>6.5</v>
       </c>
       <c r="U27" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="V27" s="15" t="n">
         <v>6</v>
-      </c>
-      <c r="V27" s="15" t="n">
-        <v>8</v>
       </c>
       <c r="W27" s="16">
         <f>$S$2*R27+$T$2*S27+$U$2*T27+$V$2*U27-$W$2*V27</f>
@@ -3144,87 +3144,87 @@
         <v>25</v>
       </c>
       <c r="B28" s="23" t="n">
-        <v>3.54</v>
+        <v>2.98</v>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>Market-making</t>
+          <t>Locked carry</t>
         </is>
       </c>
       <c r="D28" s="24" t="inlineStr">
         <is>
-          <t>Spread capture: XPLKUSDT (mexc)</t>
+          <t>Delivery basis: WLD_USDT_20260821</t>
         </is>
       </c>
       <c r="E28" s="15" t="inlineStr">
         <is>
-          <t>mexc</t>
+          <t>Gate futures</t>
         </is>
       </c>
       <c r="F28" s="16" t="n">
-        <v>1.9691</v>
+        <v>8.52</v>
       </c>
       <c r="G28" s="24" t="inlineStr">
         <is>
-          <t>% per round trip</t>
+          <t>% APR locked to expiry</t>
         </is>
       </c>
       <c r="H28" s="24" t="inlineStr">
         <is>
-          <t>minutes per RT</t>
+          <t>4.1d to delivery</t>
         </is>
       </c>
       <c r="I28" s="24" t="inlineStr">
         <is>
-          <t>10-100 fills</t>
+          <t>weekly (new contracts)</t>
         </is>
       </c>
       <c r="J28" s="25" t="n">
-        <v>500</v>
+        <v>100000</v>
       </c>
       <c r="K28" s="24" t="inlineStr">
         <is>
-          <t>live books + trade tape</t>
+          <t>mark vs spot mid</t>
         </is>
       </c>
       <c r="L28" s="15" t="n">
         <v>3</v>
       </c>
       <c r="M28" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N28" s="24" t="inlineStr">
         <is>
-          <t>INVENTORY RISK: one-sided fills accumulate positions; microcaps gap hard; sim showed +/-$90 swings vs $8 capture</t>
+          <t>Margin on short leg; locked only if held to delivery</t>
         </is>
       </c>
       <c r="O28" s="24" t="inlineStr">
         <is>
-          <t>Post maker bid+ask inside the spread (0% maker on MEXC); manage inventory</t>
+          <t>Buy spot + short dated future; converge at delivery regardless of price</t>
         </is>
       </c>
       <c r="P28" s="26" t="n">
-        <v>15</v>
+        <v>2.3</v>
       </c>
       <c r="Q28" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16 21:40 UTC</t>
+          <t>2026-08-17T04:43:00Z</t>
         </is>
       </c>
       <c r="R28" s="15" t="n">
-        <v>4.8</v>
+        <v>1.7</v>
       </c>
       <c r="S28" s="15" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="T28" s="15" t="n">
-        <v>4</v>
+        <v>7.5</v>
       </c>
       <c r="U28" s="15" t="n">
         <v>6</v>
       </c>
       <c r="V28" s="15" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="W28" s="16">
         <f>$S$2*R28+$T$2*S28+$U$2*T28+$V$2*U28-$W$2*V28</f>
@@ -3236,87 +3236,87 @@
         <v>26</v>
       </c>
       <c r="B29" s="23" t="n">
-        <v>3.51</v>
+        <v>2.98</v>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>Fixed-rate lock</t>
+          <t>Dislocation monitor</t>
         </is>
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t>Pendle PT stable yields (best liquid: 14-18% APY)</t>
+          <t>Stablecoin depeg / triangle / CEX-DEX watchlist</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>Pendle (Ethereum)</t>
+          <t>11 CEX + Jupiter + books</t>
         </is>
       </c>
       <c r="F29" s="16" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G29" s="24" t="inlineStr">
         <is>
-          <t>% APY fixed at purchase</t>
+          <t>% now; 1-30% in stress events</t>
         </is>
       </c>
       <c r="H29" s="24" t="inlineStr">
         <is>
-          <t>instant buy; hold to maturity</t>
+          <t>seconds when open</t>
         </is>
       </c>
       <c r="I29" s="24" t="inlineStr">
         <is>
-          <t>monthly (new maturities)</t>
+          <t>rare, event-driven</t>
         </is>
       </c>
       <c r="J29" s="25" t="n">
-        <v>5000000</v>
+        <v>100000</v>
       </c>
       <c r="K29" s="24" t="inlineStr">
         <is>
-          <t>Pendle API implied APY</t>
+          <t>6 scanners, order-book verified</t>
         </is>
       </c>
       <c r="L29" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M29" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N29" s="24" t="inlineStr">
         <is>
-          <t>Underlying protocol/stablecoin solvency is the paid risk; yield locked only to maturity</t>
+          <t>The USDC depeg (Mar 2023) paid 3-8% riskless for a weekend to whoever was ready; loops all negative at rest</t>
         </is>
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>Buy discounted principal token, redeem at par at maturity</t>
+          <t>Run the scanner loop; act only when it flags a verified positive</t>
         </is>
       </c>
       <c r="P29" s="26" t="n">
-        <v>4.4</v>
+        <v>0</v>
       </c>
       <c r="Q29" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16 21:40 UTC</t>
+          <t>2026-08-17 04:43 UTC</t>
         </is>
       </c>
       <c r="R29" s="15" t="n">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="S29" s="15" t="n">
         <v>3</v>
       </c>
       <c r="T29" s="15" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="U29" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V29" s="15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="W29" s="16">
         <f>$S$2*R29+$T$2*S29+$U$2*T29+$V$2*U29-$W$2*V29</f>
@@ -3328,87 +3328,87 @@
         <v>27</v>
       </c>
       <c r="B30" s="23" t="n">
-        <v>3.04</v>
+        <v>2.86</v>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>P2P fiat corridor</t>
+          <t>Locked carry</t>
         </is>
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>Ukraine in-country loop (PrivatBank both legs)</t>
+          <t>Delivery basis: UNI_USDT_20260821</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
         <is>
-          <t>OKX P2P</t>
+          <t>Gate futures</t>
         </is>
       </c>
       <c r="F30" s="16" t="n">
-        <v>2.8</v>
+        <v>6.72</v>
       </c>
       <c r="G30" s="24" t="inlineStr">
         <is>
-          <t>% per cycle</t>
+          <t>% APR locked to expiry</t>
         </is>
       </c>
       <c r="H30" s="24" t="inlineStr">
         <is>
-          <t>5-15 min per leg</t>
+          <t>4.1d to delivery</t>
         </is>
       </c>
       <c r="I30" s="24" t="inlineStr">
         <is>
-          <t>20-40</t>
+          <t>weekly (new contracts)</t>
         </is>
       </c>
       <c r="J30" s="25" t="n">
-        <v>20000</v>
+        <v>100000</v>
       </c>
       <c r="K30" s="24" t="inlineStr">
         <is>
-          <t>offer-level check incl. depth+banks</t>
-        </is>
-      </c>
-      <c r="L30" s="27" t="n">
-        <v>1</v>
+          <t>mark vs spot mid</t>
+        </is>
+      </c>
+      <c r="L30" s="15" t="n">
+        <v>3</v>
       </c>
       <c r="M30" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="N30" s="24" t="inlineStr">
+        <is>
+          <t>Margin on short leg; locked only if held to delivery</t>
+        </is>
+      </c>
+      <c r="O30" s="24" t="inlineStr">
+        <is>
+          <t>Buy spot + short dated future; converge at delivery regardless of price</t>
+        </is>
+      </c>
+      <c r="P30" s="26" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="Q30" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-17T04:43:00Z</t>
+        </is>
+      </c>
+      <c r="R30" s="15" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="S30" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="N30" s="24" t="inlineStr">
-        <is>
-          <t>REQUIRES Ukrainian bank rails - not executable from Greece; counterparty/chargeback risk</t>
-        </is>
-      </c>
-      <c r="O30" s="24" t="inlineStr">
-        <is>
-          <t>Buy USDT from merchant A, sell to merchant B, same bank transfers</t>
-        </is>
-      </c>
-      <c r="P30" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="15" t="inlineStr">
-        <is>
-          <t>2026-08-16T20:29:43Z</t>
-        </is>
-      </c>
-      <c r="R30" s="15" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="S30" s="15" t="n">
+      <c r="T30" s="15" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="U30" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="T30" s="15" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="U30" s="15" t="n">
-        <v>2</v>
-      </c>
       <c r="V30" s="15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="W30" s="16">
         <f>$S$2*R30+$T$2*S30+$U$2*T30+$V$2*U30-$W$2*V30</f>
@@ -3420,39 +3420,39 @@
         <v>28</v>
       </c>
       <c r="B31" s="23" t="n">
-        <v>2.98</v>
+        <v>2.83</v>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>Dislocation monitor</t>
+          <t>Locked carry</t>
         </is>
       </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
-          <t>Stablecoin depeg / triangle / CEX-DEX watchlist</t>
+          <t>Delivery basis: WLD_USDT_20260828</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>11 CEX + Jupiter + books</t>
+          <t>Gate futures</t>
         </is>
       </c>
       <c r="F31" s="16" t="n">
-        <v>0</v>
+        <v>5.87</v>
       </c>
       <c r="G31" s="24" t="inlineStr">
         <is>
-          <t>% now; 1-30% in stress events</t>
+          <t>% APR locked to expiry</t>
         </is>
       </c>
       <c r="H31" s="24" t="inlineStr">
         <is>
-          <t>seconds when open</t>
+          <t>11.1d to delivery</t>
         </is>
       </c>
       <c r="I31" s="24" t="inlineStr">
         <is>
-          <t>rare, event-driven</t>
+          <t>weekly (new contracts)</t>
         </is>
       </c>
       <c r="J31" s="25" t="n">
@@ -3460,35 +3460,35 @@
       </c>
       <c r="K31" s="24" t="inlineStr">
         <is>
-          <t>6 scanners, order-book verified</t>
+          <t>mark vs spot mid</t>
         </is>
       </c>
       <c r="L31" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M31" s="15" t="n">
         <v>2</v>
       </c>
       <c r="N31" s="24" t="inlineStr">
         <is>
-          <t>The USDC depeg (Mar 2023) paid 3-8% riskless for a weekend to whoever was ready; loops all negative at rest</t>
+          <t>Margin on short leg; locked only if held to delivery</t>
         </is>
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>Run the scanner loop; act only when it flags a verified positive</t>
+          <t>Buy spot + short dated future; converge at delivery regardless of price</t>
         </is>
       </c>
       <c r="P31" s="26" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="Q31" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16 21:40 UTC</t>
+          <t>2026-08-17T04:43:00Z</t>
         </is>
       </c>
       <c r="R31" s="15" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="S31" s="15" t="n">
         <v>3</v>
@@ -3497,7 +3497,7 @@
         <v>7.5</v>
       </c>
       <c r="U31" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V31" s="15" t="n">
         <v>4</v>
@@ -3512,7 +3512,7 @@
         <v>29</v>
       </c>
       <c r="B32" s="23" t="n">
-        <v>1.94</v>
+        <v>1.77</v>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
@@ -3530,7 +3530,7 @@
         </is>
       </c>
       <c r="F32" s="16" t="n">
-        <v>7.7</v>
+        <v>5.1</v>
       </c>
       <c r="G32" s="24" t="inlineStr">
         <is>
@@ -3576,11 +3576,11 @@
       </c>
       <c r="Q32" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16T14:45:46Z</t>
+          <t>2026-08-17T04:43:00Z</t>
         </is>
       </c>
       <c r="R32" s="15" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="S32" s="15" t="n">
         <v>3</v>
@@ -3859,29 +3859,29 @@
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Philadelphia Union vs. Inter Miami CF</t>
+          <t>Beşiktaş JK vs. FK Kauno Žalgiris</t>
         </is>
       </c>
       <c r="B2" s="29" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="29" t="n">
-        <v>1.03</v>
+        <v>1.012</v>
       </c>
       <c r="D2" s="29" t="n">
-        <v>0.03</v>
+        <v>0.012</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>1.97</v>
+        <v>1.988</v>
       </c>
       <c r="F2" s="29" t="n">
-        <v>1.523</v>
+        <v>0.604</v>
       </c>
       <c r="G2" s="29" t="n">
-        <v>67.3</v>
+        <v>5</v>
       </c>
       <c r="H2" s="29" t="n">
-        <v>2.02</v>
+        <v>0.06</v>
       </c>
       <c r="I2" s="29" t="inlineStr">
         <is>
@@ -3899,22 +3899,22 @@
         <v>3</v>
       </c>
       <c r="C3" s="29" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="D3" s="29" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>1.98</v>
+        <v>1.99</v>
       </c>
       <c r="F3" s="29" t="n">
-        <v>1.01</v>
+        <v>0.503</v>
       </c>
       <c r="G3" s="29" t="n">
-        <v>63.1</v>
+        <v>58.1</v>
       </c>
       <c r="H3" s="29" t="n">
-        <v>1.26</v>
+        <v>0.58</v>
       </c>
       <c r="I3" s="29" t="inlineStr">
         <is>
@@ -3925,62 +3925,50 @@
     <row r="4">
       <c r="A4" s="29" t="inlineStr">
         <is>
-          <t>GPU rental prices (H100) end of August?</t>
+          <t>Pro Football: AFC South Champion</t>
         </is>
       </c>
       <c r="B4" s="29" t="n">
-        <v>6</v>
-      </c>
-      <c r="C4" s="29" t="n">
-        <v>1.013</v>
-      </c>
-      <c r="D4" s="29" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="E4" s="29" t="n">
-        <v>4.987</v>
-      </c>
-      <c r="F4" s="29" t="n">
-        <v>0.261</v>
-      </c>
-      <c r="G4" s="29" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="H4" s="29" t="n">
-        <v>0.34</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C4" s="29" t="n"/>
+      <c r="D4" s="29" t="n"/>
+      <c r="E4" s="29" t="n"/>
+      <c r="F4" s="29" t="n"/>
+      <c r="G4" s="29" t="n"/>
+      <c r="H4" s="29" t="n"/>
       <c r="I4" s="29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>book_unavailable</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>Anthropic IPO Closing Market Cap</t>
+          <t>Al Ta'ee Saudi Club vs. Al Qadisiyah Saudi Club</t>
         </is>
       </c>
       <c r="B5" s="29" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C5" s="29" t="n">
-        <v>1.022</v>
+        <v>1.007</v>
       </c>
       <c r="D5" s="29" t="n">
-        <v>0.022</v>
+        <v>0.007</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>8.978</v>
+        <v>1.993</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.245</v>
+        <v>0.351</v>
       </c>
       <c r="G5" s="29" t="n">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="H5" s="29" t="n">
-        <v>0.14</v>
+        <v>0</v>
       </c>
       <c r="I5" s="29" t="inlineStr">
         <is>
@@ -3991,11 +3979,11 @@
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>GPU rental prices (H200) end of August?</t>
+          <t>Fed Decision in December?</t>
         </is>
       </c>
       <c r="B6" s="29" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6" s="29" t="n">
         <v>1.01</v>
@@ -4004,16 +3992,16 @@
         <v>0.01</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>4.99</v>
+        <v>3.99</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.2</v>
+        <v>0.251</v>
       </c>
       <c r="G6" s="29" t="n">
-        <v>30</v>
+        <v>782</v>
       </c>
       <c r="H6" s="29" t="n">
-        <v>0.3</v>
+        <v>7.82</v>
       </c>
       <c r="I6" s="29" t="inlineStr">
         <is>
@@ -4024,29 +4012,29 @@
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>James Fishback vote share in 2026 Florida Republican Governor Primary?</t>
+          <t>Highest temperature in Buenos Aires on August 18?</t>
         </is>
       </c>
       <c r="B7" s="29" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C7" s="29" t="n">
-        <v>1.009</v>
+        <v>1.024</v>
       </c>
       <c r="D7" s="29" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.024</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>4.991</v>
+        <v>9.976000000000001</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>0.18</v>
+        <v>0.241</v>
       </c>
       <c r="G7" s="29" t="n">
-        <v>19.9</v>
+        <v>4</v>
       </c>
       <c r="H7" s="29" t="n">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="I7" s="29" t="inlineStr">
         <is>
@@ -4064,22 +4052,22 @@
         <v>5</v>
       </c>
       <c r="C8" s="29" t="n">
-        <v>1.007</v>
+        <v>1.009</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>0.007</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>3.993</v>
+        <v>3.991</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.175</v>
+        <v>0.226</v>
       </c>
       <c r="G8" s="29" t="n">
         <v>100</v>
       </c>
       <c r="H8" s="29" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="I8" s="29" t="inlineStr">
         <is>
@@ -4090,62 +4078,50 @@
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>Fed Decision in December?</t>
+          <t xml:space="preserve">Pro Football: NFC West Champion  </t>
         </is>
       </c>
       <c r="B9" s="29" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="29" t="n">
-        <v>1.007</v>
-      </c>
-      <c r="D9" s="29" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="E9" s="29" t="n">
-        <v>3.993</v>
-      </c>
-      <c r="F9" s="29" t="n">
-        <v>0.175</v>
-      </c>
-      <c r="G9" s="29" t="n">
-        <v>835</v>
-      </c>
-      <c r="H9" s="29" t="n">
-        <v>5.84</v>
-      </c>
+      <c r="C9" s="29" t="n"/>
+      <c r="D9" s="29" t="n"/>
+      <c r="E9" s="29" t="n"/>
+      <c r="F9" s="29" t="n"/>
+      <c r="G9" s="29" t="n"/>
+      <c r="H9" s="29" t="n"/>
       <c r="I9" s="29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>book_unavailable</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
         <is>
-          <t>Fed Decision in December?</t>
+          <t>Anthropic IPO Closing Market Cap</t>
         </is>
       </c>
       <c r="B10" s="29" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C10" s="29" t="n">
-        <v>1.007</v>
+        <v>1.016</v>
       </c>
       <c r="D10" s="29" t="n">
-        <v>0.007</v>
+        <v>0.016</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>3.993</v>
+        <v>8.984</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>0.175</v>
+        <v>0.178</v>
       </c>
       <c r="G10" s="29" t="n">
-        <v>835</v>
+        <v>40</v>
       </c>
       <c r="H10" s="29" t="n">
-        <v>5.84</v>
+        <v>0.64</v>
       </c>
       <c r="I10" s="29" t="inlineStr">
         <is>
@@ -4156,29 +4132,29 @@
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>Private Companies - greatest valuation growth August 2026</t>
+          <t>Highest temperature in Warsaw on August 17?</t>
         </is>
       </c>
       <c r="B11" s="29" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C11" s="29" t="n">
-        <v>1.007</v>
+        <v>1.021</v>
       </c>
       <c r="D11" s="29" t="n">
-        <v>0.007</v>
+        <v>0.021</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>3.993</v>
+        <v>9.978999999999999</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>0.175</v>
+        <v>0.21</v>
       </c>
       <c r="G11" s="29" t="n">
-        <v>21.3</v>
+        <v>2</v>
       </c>
       <c r="H11" s="29" t="n">
-        <v>0.15</v>
+        <v>0.04</v>
       </c>
       <c r="I11" s="29" t="inlineStr">
         <is>
@@ -4189,77 +4165,53 @@
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
-          <t>Highest temperature in Ankara on August 18?</t>
+          <t>Los Angeles Mayoral Election</t>
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>11</v>
-      </c>
-      <c r="C12" s="29" t="n">
-        <v>1.017</v>
-      </c>
-      <c r="D12" s="29" t="n">
-        <v>0.017</v>
-      </c>
-      <c r="E12" s="29" t="n">
-        <v>9.983000000000001</v>
-      </c>
-      <c r="F12" s="29" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="G12" s="29" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="H12" s="29" t="n">
-        <v>0.1</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="29" t="n"/>
+      <c r="F12" s="29" t="n"/>
+      <c r="G12" s="29" t="n"/>
+      <c r="H12" s="29" t="n"/>
       <c r="I12" s="29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>book_unavailable</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>Highest temperature in Warsaw on August 18?</t>
+          <t>NBA: 2027 Eastern Conference Champion</t>
         </is>
       </c>
       <c r="B13" s="29" t="n">
-        <v>11</v>
-      </c>
-      <c r="C13" s="29" t="n">
-        <v>1.016</v>
-      </c>
-      <c r="D13" s="29" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="E13" s="29" t="n">
-        <v>9.984</v>
-      </c>
-      <c r="F13" s="29" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="G13" s="29" t="n">
-        <v>5</v>
-      </c>
-      <c r="H13" s="29" t="n">
-        <v>0.08</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="29" t="n"/>
+      <c r="F13" s="29" t="n"/>
+      <c r="G13" s="29" t="n"/>
+      <c r="H13" s="29" t="n"/>
       <c r="I13" s="29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>book_unavailable</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>NBA: 2027 Eastern Conference Champion</t>
+          <t>Pro Football: 2027 Champion</t>
         </is>
       </c>
       <c r="B14" s="29" t="n">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="C14" s="29" t="n"/>
       <c r="D14" s="29" t="n"/>
@@ -4276,11 +4228,11 @@
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>NHL: 2027 Western Conference Champion</t>
+          <t>LCK 2026 Season Winner</t>
         </is>
       </c>
       <c r="B15" s="29" t="n">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="C15" s="29" t="n"/>
       <c r="D15" s="29" t="n"/>
@@ -4355,11 +4307,11 @@
       </c>
       <c r="C2" s="29" t="inlineStr">
         <is>
-          <t>4.7d, spot 0.3448 fut 0.3476</t>
+          <t>4.1d, spot 0.36265000000000003 fut 0.363</t>
         </is>
       </c>
       <c r="D2" s="29" t="n">
-        <v>62.82</v>
+        <v>8.52</v>
       </c>
       <c r="E2" s="29" t="inlineStr">
         <is>
@@ -4380,11 +4332,11 @@
       </c>
       <c r="C3" s="29" t="inlineStr">
         <is>
-          <t>4.7d, spot 3.2714999999999996 fut 3.288</t>
+          <t>4.1d, spot 3.2824999999999998 fut 3.285</t>
         </is>
       </c>
       <c r="D3" s="29" t="n">
-        <v>39.02</v>
+        <v>6.72</v>
       </c>
       <c r="E3" s="29" t="inlineStr">
         <is>
@@ -4400,16 +4352,16 @@
       </c>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>AVAX_USDT_20260821</t>
+          <t>WLD_USDT_20260828</t>
         </is>
       </c>
       <c r="C4" s="29" t="inlineStr">
         <is>
-          <t>4.7d, spot 6.3785 fut 6.41</t>
+          <t>11.1d, spot 0.36265000000000003 fut 0.3633</t>
         </is>
       </c>
       <c r="D4" s="29" t="n">
-        <v>38.21</v>
+        <v>5.87</v>
       </c>
       <c r="E4" s="29" t="inlineStr">
         <is>
@@ -4425,16 +4377,16 @@
       </c>
       <c r="B5" s="29" t="inlineStr">
         <is>
-          <t>WLD_USDT_20260828</t>
+          <t>BTC_USDT_20260828</t>
         </is>
       </c>
       <c r="C5" s="29" t="inlineStr">
         <is>
-          <t>11.7d, spot 0.3448 fut 0.348</t>
+          <t>11.1d, spot 63507.850000000006 fut 63608.75</t>
         </is>
       </c>
       <c r="D5" s="29" t="n">
-        <v>28.91</v>
+        <v>5.21</v>
       </c>
       <c r="E5" s="29" t="inlineStr">
         <is>
@@ -4455,11 +4407,11 @@
       </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>4.7d, spot 9.3215 fut 9.352</t>
+          <t>4.1d, spot 9.473500000000001 fut 9.479</t>
         </is>
       </c>
       <c r="D6" s="29" t="n">
-        <v>25.31</v>
+        <v>5.12</v>
       </c>
       <c r="E6" s="29" t="inlineStr">
         <is>
@@ -4475,16 +4427,16 @@
       </c>
       <c r="B7" s="29" t="inlineStr">
         <is>
-          <t>UNI_USDT_20260828</t>
+          <t>LINK_USDT_20260828</t>
         </is>
       </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
-          <t>11.7d, spot 3.2714999999999996 fut 3.292</t>
+          <t>11.1d, spot 9.473500000000001 fut 9.488</t>
         </is>
       </c>
       <c r="D7" s="29" t="n">
-        <v>19.52</v>
+        <v>5.02</v>
       </c>
       <c r="E7" s="29" t="inlineStr">
         <is>
@@ -4500,16 +4452,16 @@
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
-          <t>AVAX_USDT_20260828</t>
+          <t>DOGE_USDT_20261225</t>
         </is>
       </c>
       <c r="C8" s="29" t="inlineStr">
         <is>
-          <t>11.7d, spot 6.3785 fut 6.417</t>
+          <t>130.1d, spot 0.07022500000000001 fut 0.07144</t>
         </is>
       </c>
       <c r="D8" s="29" t="n">
-        <v>18.8</v>
+        <v>4.85</v>
       </c>
       <c r="E8" s="29" t="inlineStr">
         <is>
@@ -4525,16 +4477,16 @@
       </c>
       <c r="B9" s="29" t="inlineStr">
         <is>
-          <t>LTC_USDT_20260821</t>
+          <t>ETH_USDT_20260821</t>
         </is>
       </c>
       <c r="C9" s="29" t="inlineStr">
         <is>
-          <t>4.7d, spot 44.275000000000006 fut 44.36</t>
+          <t>4.1d, spot 1902.8249999999998 fut 1903.85</t>
         </is>
       </c>
       <c r="D9" s="29" t="n">
-        <v>14.85</v>
+        <v>4.75</v>
       </c>
       <c r="E9" s="29" t="inlineStr">
         <is>
@@ -4550,16 +4502,16 @@
       </c>
       <c r="B10" s="29" t="inlineStr">
         <is>
-          <t>LINK_USDT_20260828</t>
+          <t>UNI_USDT_20260828</t>
         </is>
       </c>
       <c r="C10" s="29" t="inlineStr">
         <is>
-          <t>11.7d, spot 9.3215 fut 9.361</t>
+          <t>11.1d, spot 3.2824999999999998 fut 3.287</t>
         </is>
       </c>
       <c r="D10" s="29" t="n">
-        <v>13.2</v>
+        <v>4.49</v>
       </c>
       <c r="E10" s="29" t="inlineStr">
         <is>
@@ -4575,16 +4527,16 @@
       </c>
       <c r="B11" s="29" t="inlineStr">
         <is>
-          <t>DOGE_USDT_20260821</t>
+          <t>BTC_USDT_20261225</t>
         </is>
       </c>
       <c r="C11" s="29" t="inlineStr">
         <is>
-          <t>4.7d, spot 0.069925 fut 0.07002</t>
+          <t>130.1d, spot 63507.850000000006 fut 64517.15</t>
         </is>
       </c>
       <c r="D11" s="29" t="n">
-        <v>10.51</v>
+        <v>4.46</v>
       </c>
       <c r="E11" s="29" t="inlineStr">
         <is>
@@ -4600,16 +4552,16 @@
       </c>
       <c r="B12" s="29" t="inlineStr">
         <is>
-          <t>LTC_USDT_20260828</t>
+          <t>DOGE_USDT_20260925</t>
         </is>
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
-          <t>11.7d, spot 44.275000000000006 fut 44.4</t>
+          <t>39.1d, spot 0.07022500000000001 fut 0.07056</t>
         </is>
       </c>
       <c r="D12" s="29" t="n">
-        <v>8.789999999999999</v>
+        <v>4.45</v>
       </c>
       <c r="E12" s="29" t="inlineStr">
         <is>
@@ -4625,16 +4577,16 @@
       </c>
       <c r="B13" s="29" t="inlineStr">
         <is>
-          <t>BTC_USDT_20260821</t>
+          <t>BTC_USDT_20260925</t>
         </is>
       </c>
       <c r="C13" s="29" t="inlineStr">
         <is>
-          <t>4.7d, spot 63065.55 fut 63134.82</t>
+          <t>39.1d, spot 63507.850000000006 fut 63801.5</t>
         </is>
       </c>
       <c r="D13" s="29" t="n">
-        <v>8.5</v>
+        <v>4.31</v>
       </c>
       <c r="E13" s="29" t="inlineStr">
         <is>
@@ -4650,16 +4602,16 @@
       </c>
       <c r="B14" s="29" t="inlineStr">
         <is>
-          <t>ADA_USDT_20260821</t>
+          <t>LTC_USDT_20260828</t>
         </is>
       </c>
       <c r="C14" s="29" t="inlineStr">
         <is>
-          <t>4.7d, spot 0.176375 fut 0.1762</t>
+          <t>11.1d, spot 44.285 fut 44.34</t>
         </is>
       </c>
       <c r="D14" s="29" t="n">
-        <v>-7.68</v>
+        <v>4.07</v>
       </c>
       <c r="E14" s="29" t="inlineStr">
         <is>
@@ -4675,16 +4627,16 @@
       </c>
       <c r="B15" s="29" t="inlineStr">
         <is>
-          <t>ETH_USDT_20260821</t>
+          <t>BTC_USDT_20260821</t>
         </is>
       </c>
       <c r="C15" s="29" t="inlineStr">
         <is>
-          <t>4.7d, spot 1881.705 fut 1883.54</t>
+          <t>4.1d, spot 63507.850000000006 fut 63536.9</t>
         </is>
       </c>
       <c r="D15" s="29" t="n">
-        <v>7.54</v>
+        <v>4.04</v>
       </c>
       <c r="E15" s="29" t="inlineStr">
         <is>
@@ -4700,16 +4652,16 @@
       </c>
       <c r="B16" s="29" t="inlineStr">
         <is>
-          <t>DOGE_USDT_20260828</t>
+          <t>ETH_USDT_20260828</t>
         </is>
       </c>
       <c r="C16" s="29" t="inlineStr">
         <is>
-          <t>11.7d, spot 0.069925 fut 0.07009</t>
+          <t>11.1d, spot 1902.8249999999998 fut 1905.06</t>
         </is>
       </c>
       <c r="D16" s="29" t="n">
-        <v>7.35</v>
+        <v>3.85</v>
       </c>
       <c r="E16" s="29" t="inlineStr">
         <is>
@@ -4734,7 +4686,7 @@
         </is>
       </c>
       <c r="D17" s="29" t="n">
-        <v>1.521</v>
+        <v>3.166</v>
       </c>
       <c r="E17" s="29" t="inlineStr">
         <is>
@@ -4759,7 +4711,7 @@
         </is>
       </c>
       <c r="D18" s="29" t="n">
-        <v>1.379</v>
+        <v>1.033</v>
       </c>
       <c r="E18" s="29" t="inlineStr">
         <is>
@@ -4784,7 +4736,7 @@
         </is>
       </c>
       <c r="D19" s="29" t="n">
-        <v>1.295</v>
+        <v>0.714</v>
       </c>
       <c r="E19" s="29" t="inlineStr">
         <is>
@@ -4800,16 +4752,16 @@
       </c>
       <c r="B20" s="29" t="inlineStr">
         <is>
-          <t>COTI</t>
+          <t>LUMIA</t>
         </is>
       </c>
       <c r="C20" s="29" t="inlineStr">
         <is>
-          <t>long gate short bitget</t>
+          <t>long bitget short gate</t>
         </is>
       </c>
       <c r="D20" s="29" t="n">
-        <v>1.216</v>
+        <v>0.681</v>
       </c>
       <c r="E20" s="29" t="inlineStr">
         <is>
@@ -4825,7 +4777,7 @@
       </c>
       <c r="B21" s="29" t="inlineStr">
         <is>
-          <t>ALICE</t>
+          <t>STABLE</t>
         </is>
       </c>
       <c r="C21" s="29" t="inlineStr">
@@ -4834,7 +4786,7 @@
         </is>
       </c>
       <c r="D21" s="29" t="n">
-        <v>1.123</v>
+        <v>0.667</v>
       </c>
       <c r="E21" s="29" t="inlineStr">
         <is>
@@ -4850,7 +4802,7 @@
       </c>
       <c r="B22" s="29" t="inlineStr">
         <is>
-          <t>BICO</t>
+          <t>STEEM</t>
         </is>
       </c>
       <c r="C22" s="29" t="inlineStr">
@@ -4859,7 +4811,7 @@
         </is>
       </c>
       <c r="D22" s="29" t="n">
-        <v>0.734</v>
+        <v>0.634</v>
       </c>
       <c r="E22" s="29" t="inlineStr">
         <is>
@@ -4875,16 +4827,16 @@
       </c>
       <c r="B23" s="29" t="inlineStr">
         <is>
-          <t>COW</t>
+          <t>POWER</t>
         </is>
       </c>
       <c r="C23" s="29" t="inlineStr">
         <is>
-          <t>long gate short bitget</t>
+          <t>long bitget short gate</t>
         </is>
       </c>
       <c r="D23" s="29" t="n">
-        <v>0.707</v>
+        <v>0.624</v>
       </c>
       <c r="E23" s="29" t="inlineStr">
         <is>
@@ -4900,16 +4852,16 @@
       </c>
       <c r="B24" s="29" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
-          <t>long bitget short gate</t>
+          <t>long gate short bitget</t>
         </is>
       </c>
       <c r="D24" s="29" t="n">
-        <v>0.553</v>
+        <v>0.549</v>
       </c>
       <c r="E24" s="29" t="inlineStr">
         <is>
@@ -4925,7 +4877,7 @@
       </c>
       <c r="B25" s="29" t="inlineStr">
         <is>
-          <t>XAI</t>
+          <t>ALICE</t>
         </is>
       </c>
       <c r="C25" s="29" t="inlineStr">
@@ -4934,7 +4886,7 @@
         </is>
       </c>
       <c r="D25" s="29" t="n">
-        <v>0.441</v>
+        <v>0.546</v>
       </c>
       <c r="E25" s="29" t="inlineStr">
         <is>
@@ -4950,7 +4902,7 @@
       </c>
       <c r="B26" s="29" t="inlineStr">
         <is>
-          <t>RAVE</t>
+          <t>RESOLV</t>
         </is>
       </c>
       <c r="C26" s="29" t="inlineStr">
@@ -4959,7 +4911,7 @@
         </is>
       </c>
       <c r="D26" s="29" t="n">
-        <v>0.435</v>
+        <v>0.505</v>
       </c>
       <c r="E26" s="29" t="inlineStr">
         <is>
@@ -4975,16 +4927,16 @@
       </c>
       <c r="B27" s="29" t="inlineStr">
         <is>
-          <t>ESPORTS</t>
+          <t>COTI</t>
         </is>
       </c>
       <c r="C27" s="29" t="inlineStr">
         <is>
-          <t>long bitget short gate</t>
+          <t>long gate short bitget</t>
         </is>
       </c>
       <c r="D27" s="29" t="n">
-        <v>0.423</v>
+        <v>0.47</v>
       </c>
       <c r="E27" s="29" t="inlineStr">
         <is>
@@ -5000,16 +4952,16 @@
       </c>
       <c r="B28" s="29" t="inlineStr">
         <is>
-          <t>TAC</t>
+          <t>DEXE</t>
         </is>
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>long bitget short gate</t>
+          <t>long gate short bitget</t>
         </is>
       </c>
       <c r="D28" s="29" t="n">
-        <v>0.333</v>
+        <v>0.438</v>
       </c>
       <c r="E28" s="29" t="inlineStr">
         <is>
@@ -5025,16 +4977,16 @@
       </c>
       <c r="B29" s="29" t="inlineStr">
         <is>
-          <t>ARKM</t>
+          <t>COW</t>
         </is>
       </c>
       <c r="C29" s="29" t="inlineStr">
         <is>
-          <t>long bitget short gate</t>
+          <t>long gate short bitget</t>
         </is>
       </c>
       <c r="D29" s="29" t="n">
-        <v>0.33</v>
+        <v>0.412</v>
       </c>
       <c r="E29" s="29" t="inlineStr">
         <is>
@@ -5050,7 +5002,7 @@
       </c>
       <c r="B30" s="29" t="inlineStr">
         <is>
-          <t>AIN</t>
+          <t>CVC</t>
         </is>
       </c>
       <c r="C30" s="29" t="inlineStr">
@@ -5059,7 +5011,7 @@
         </is>
       </c>
       <c r="D30" s="29" t="n">
-        <v>0.306</v>
+        <v>0.403</v>
       </c>
       <c r="E30" s="29" t="inlineStr">
         <is>
@@ -5075,16 +5027,16 @@
       </c>
       <c r="B31" s="29" t="inlineStr">
         <is>
-          <t>PROM</t>
+          <t>NAORIS</t>
         </is>
       </c>
       <c r="C31" s="29" t="inlineStr">
         <is>
-          <t>long gate short bitget</t>
+          <t>long bitget short gate</t>
         </is>
       </c>
       <c r="D31" s="29" t="n">
-        <v>0.297</v>
+        <v>0.401</v>
       </c>
       <c r="E31" s="29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Loop refresh: sweeps + new-sectors rescan
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0131Tm9QwYyPuHrkNkGr7Vys
</commit_message>
<xml_diff>
--- a/arb-scanner/data/Arbitrage_Ledger.xlsx
+++ b/arb-scanner/data/Arbitrage_Ledger.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-17 04:43 UTC from six live scanners: 11 crypto exchanges (~9,500 pairs), Polymarket + Kalshi order books,</t>
+          <t>Generated 2026-08-17 08:42 UTC from six live scanners: 11 crypto exchanges (~9,500 pairs), Polymarket + Kalshi order books,</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>2026-08-17 04:43 UTC</t>
+          <t>2026-08-17 08:42 UTC</t>
         </is>
       </c>
       <c r="R4" s="15" t="n">
@@ -1304,7 +1304,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="10" t="n">
-        <v>4.25</v>
+        <v>4.26</v>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="J8" s="13" t="n">
-        <v>3120</v>
+        <v>3300</v>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>2026-08-17T04:42:19Z</t>
+          <t>2026-08-17T08:41:52Z</t>
         </is>
       </c>
       <c r="R8" s="15" t="n">
@@ -1378,7 +1378,7 @@
         <v>6</v>
       </c>
       <c r="T8" s="15" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="U8" s="15" t="n">
         <v>8</v>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>2026-08-17T04:42:19Z</t>
+          <t>2026-08-17T08:41:52Z</t>
         </is>
       </c>
       <c r="R9" s="15" t="n">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>2026-08-17T04:42:19Z</t>
+          <t>2026-08-17T08:41:52Z</t>
         </is>
       </c>
       <c r="R10" s="15" t="n">
@@ -1580,7 +1580,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="10" t="n">
-        <v>3.93</v>
+        <v>4.01</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: Beşiktaş JK vs. FK Kauno Žalgiris</t>
+          <t>Neg-risk sweep: How many Fed rate cuts in 2026?</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -1598,7 +1598,7 @@
         </is>
       </c>
       <c r="F11" s="12" t="n">
-        <v>0.604</v>
+        <v>0.075</v>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
@@ -1616,7 +1616,7 @@
         </is>
       </c>
       <c r="J11" s="13" t="n">
-        <v>10</v>
+        <v>9419</v>
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
@@ -1636,25 +1636,25 @@
       </c>
       <c r="O11" s="11" t="inlineStr">
         <is>
-          <t>Buy NO on all 3 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
+          <t>Buy NO on all 13 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P11" s="14" t="n">
-        <v>0.5</v>
+        <v>20</v>
       </c>
       <c r="Q11" s="9" t="inlineStr">
         <is>
-          <t>2026-08-17T04:42:19Z</t>
+          <t>2026-08-17T08:41:52Z</t>
         </is>
       </c>
       <c r="R11" s="15" t="n">
-        <v>3.7</v>
+        <v>1.7</v>
       </c>
       <c r="S11" s="15" t="n">
         <v>6</v>
       </c>
       <c r="T11" s="15" t="n">
-        <v>1.5</v>
+        <v>6</v>
       </c>
       <c r="U11" s="15" t="n">
         <v>8</v>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="F12" s="20" t="n">
-        <v>8.1</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="J12" s="21" t="n">
-        <v>5115081</v>
+        <v>5154799</v>
       </c>
       <c r="K12" s="19" t="inlineStr">
         <is>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="O12" s="19" t="inlineStr">
         <is>
-          <t>Borrow WETH at 0% on compound-v3, lend at 8.1% on fusion-by-ipor</t>
+          <t>Borrow WETH at 0% on compound-v3, lend at 8.13% on fusion-by-ipor</t>
         </is>
       </c>
       <c r="P12" s="22" t="n">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="Q12" s="17" t="inlineStr">
         <is>
-          <t>2026-08-16T20:29:43Z</t>
+          <t>2026-08-17T08:42:10Z</t>
         </is>
       </c>
       <c r="R12" s="15" t="n">
@@ -1764,34 +1764,34 @@
         <v>10</v>
       </c>
       <c r="B13" s="18" t="n">
-        <v>3.9</v>
+        <v>3.93</v>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>Rate arbitrage</t>
+          <t>DeFi rate arbitrage</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>EURC on-chain vs Greek deposit</t>
+          <t>Borrow-lend spread: SUSDAT on Ethereum</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
-          <t>Aave v3 Ethereum</t>
+          <t>morpho-blue -&gt; saturn</t>
         </is>
       </c>
       <c r="F13" s="20" t="n">
-        <v>2.6</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>% per year net of bank rate</t>
+          <t>% per year on borrowed notional</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>instant</t>
+          <t>instant entry/exit</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
@@ -1800,39 +1800,39 @@
         </is>
       </c>
       <c r="J13" s="21" t="n">
-        <v>11000000</v>
+        <v>9807046</v>
       </c>
       <c r="K13" s="19" t="inlineStr">
         <is>
-          <t>DefiLlama: EURC 2.93% APY, $11M TVL</t>
+          <t>DefiLlama live rates</t>
         </is>
       </c>
       <c r="L13" s="17" t="n">
         <v>3</v>
       </c>
       <c r="M13" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Smart-contract + stablecoin issuer risk; beats ESTR slightly</t>
+          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
         </is>
       </c>
       <c r="O13" s="19" t="inlineStr">
         <is>
-          <t>Hold EURC, supply on Aave</t>
+          <t>Borrow SUSDAT at 10.36% on morpho-blue, lend at 18.4% on saturn</t>
         </is>
       </c>
       <c r="P13" s="22" t="n">
-        <v>0.7</v>
+        <v>1.5</v>
       </c>
       <c r="Q13" s="17" t="inlineStr">
         <is>
-          <t>2026-08-17 04:43 UTC</t>
+          <t>2026-08-17T08:42:10Z</t>
         </is>
       </c>
       <c r="R13" s="15" t="n">
-        <v>0.5</v>
+        <v>1.6</v>
       </c>
       <c r="S13" s="15" t="n">
         <v>9</v>
@@ -1844,7 +1844,7 @@
         <v>6</v>
       </c>
       <c r="V13" s="15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W13" s="16">
         <f>$S$2*R13+$T$2*S13+$U$2*T13+$V$2*U13-$W$2*V13</f>
@@ -1856,87 +1856,87 @@
         <v>11</v>
       </c>
       <c r="B14" s="18" t="n">
-        <v>3.87</v>
+        <v>3.91</v>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Gaming items</t>
+          <t>Prediction structural</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>CS2 skins spend-discount (median 22.1% off Steam)</t>
+          <t>Neg-risk sweep: Beşiktaş JK vs. FK Kauno Žalgiris</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
-          <t>Skinport -&gt; Steam ecosystem</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="F14" s="20" t="n">
-        <v>22.1</v>
+        <v>0.553</v>
       </c>
       <c r="G14" s="19" t="inlineStr">
         <is>
-          <t>% discount on Steam spend</t>
+          <t>% per cycle (riskless)</t>
         </is>
       </c>
       <c r="H14" s="19" t="inlineStr">
         <is>
-          <t>instant</t>
+          <t>minutes</t>
         </is>
       </c>
       <c r="I14" s="19" t="inlineStr">
         <is>
-          <t>unlimited for own spending</t>
+          <t>5-20 (as books refill)</t>
         </is>
       </c>
       <c r="J14" s="21" t="n">
-        <v>1000</v>
+        <v>10</v>
       </c>
       <c r="K14" s="19" t="inlineStr">
         <is>
-          <t>full 21k-item catalog</t>
+          <t>live CLOB, every outcome book</t>
         </is>
       </c>
       <c r="L14" s="17" t="n">
         <v>4</v>
       </c>
       <c r="M14" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>ONE-WAY: Steam wallet cannot cash out - only worth it for money you'd spend on Steam anyway</t>
+          <t>Depth-capped; edge locked at fill; no-fee venue</t>
         </is>
       </c>
       <c r="O14" s="19" t="inlineStr">
         <is>
-          <t>Buy discounted items on Skinport instead of paying Steam prices</t>
+          <t>Buy NO on all 3 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P14" s="22" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="Q14" s="17" t="inlineStr">
         <is>
-          <t>2026-08-16T20:29:43Z</t>
+          <t>2026-08-17T08:41:52Z</t>
         </is>
       </c>
       <c r="R14" s="15" t="n">
-        <v>5.5</v>
+        <v>3.6</v>
       </c>
       <c r="S14" s="15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="T14" s="15" t="n">
-        <v>4.5</v>
+        <v>1.5</v>
       </c>
       <c r="U14" s="15" t="n">
         <v>8</v>
       </c>
       <c r="V14" s="15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W14" s="16">
         <f>$S$2*R14+$T$2*S14+$U$2*T14+$V$2*U14-$W$2*V14</f>
@@ -1948,87 +1948,87 @@
         <v>12</v>
       </c>
       <c r="B15" s="18" t="n">
-        <v>3.82</v>
+        <v>3.9</v>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>Prediction structural</t>
+          <t>Rate arbitrage</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Ladder violation: Will Solana reach $320 by December 31, 2</t>
+          <t>EURC on-chain vs Greek deposit</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Aave v3 Ethereum</t>
         </is>
       </c>
       <c r="F15" s="20" t="n">
-        <v>1.11</v>
+        <v>2.6</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>% locked at fill</t>
+          <t>% per year net of bank rate</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>instant fill; pays at resolution</t>
+          <t>instant</t>
         </is>
       </c>
       <c r="I15" s="19" t="inlineStr">
         <is>
-          <t>when flagged (few/week)</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="J15" s="21" t="n">
-        <v>50</v>
+        <v>11000000</v>
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>live CLOB depth</t>
+          <t>DefiLlama: EURC 2.93% APY, $11M TVL</t>
         </is>
       </c>
       <c r="L15" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="M15" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N15" s="19" t="inlineStr">
+        <is>
+          <t>Smart-contract + stablecoin issuer risk; beats ESTR slightly</t>
+        </is>
+      </c>
+      <c r="O15" s="19" t="inlineStr">
+        <is>
+          <t>Hold EURC, supply on Aave</t>
+        </is>
+      </c>
+      <c r="P15" s="22" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Q15" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-17 08:42 UTC</t>
+        </is>
+      </c>
+      <c r="R15" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S15" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="T15" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="U15" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="V15" s="15" t="n">
         <v>4</v>
-      </c>
-      <c r="M15" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="N15" s="19" t="inlineStr">
-        <is>
-          <t>Riskless at fill; capital returns at event resolution; ~$50 size</t>
-        </is>
-      </c>
-      <c r="O15" s="19" t="inlineStr">
-        <is>
-          <t>Buy YES weaker strike + NO stronger strike for &lt; $1/set; min payout $1, $2 if between strikes</t>
-        </is>
-      </c>
-      <c r="P15" s="22" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q15" s="17" t="inlineStr">
-        <is>
-          <t>2026-08-17T04:43:00Z</t>
-        </is>
-      </c>
-      <c r="R15" s="15" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="S15" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="T15" s="15" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="U15" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="V15" s="15" t="n">
-        <v>2</v>
       </c>
       <c r="W15" s="16">
         <f>$S$2*R15+$T$2*S15+$U$2*T15+$V$2*U15-$W$2*V15</f>
@@ -2040,87 +2040,87 @@
         <v>13</v>
       </c>
       <c r="B16" s="18" t="n">
-        <v>3.82</v>
+        <v>3.88</v>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>DeFi rate arbitrage</t>
+          <t>Prediction structural</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Borrow-lend spread: USD3 on Ethereum</t>
+          <t>Neg-risk sweep: Anthropic IPO Closing Market Cap</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>morpho-blue -&gt; pendle</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="F16" s="20" t="n">
-        <v>7.12</v>
+        <v>0.189</v>
       </c>
       <c r="G16" s="19" t="inlineStr">
         <is>
-          <t>% per year on borrowed notional</t>
+          <t>% per cycle (riskless)</t>
         </is>
       </c>
       <c r="H16" s="19" t="inlineStr">
         <is>
-          <t>instant entry/exit</t>
+          <t>minutes</t>
         </is>
       </c>
       <c r="I16" s="19" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>5-20 (as books refill)</t>
         </is>
       </c>
       <c r="J16" s="21" t="n">
-        <v>2763264</v>
+        <v>171</v>
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>DefiLlama live rates</t>
+          <t>live CLOB, every outcome book</t>
         </is>
       </c>
       <c r="L16" s="17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M16" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
+          <t>Depth-capped; edge locked at fill; no-fee venue</t>
         </is>
       </c>
       <c r="O16" s="19" t="inlineStr">
         <is>
-          <t>Borrow USD3 at 7.27% on morpho-blue, lend at 14.39% on pendle</t>
+          <t>Buy NO on all 10 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P16" s="22" t="n">
-        <v>1.4</v>
+        <v>2.6</v>
       </c>
       <c r="Q16" s="17" t="inlineStr">
         <is>
-          <t>2026-08-16T20:29:43Z</t>
+          <t>2026-08-17T08:41:52Z</t>
         </is>
       </c>
       <c r="R16" s="15" t="n">
-        <v>1.4</v>
+        <v>2.6</v>
       </c>
       <c r="S16" s="15" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="T16" s="15" t="n">
-        <v>9.699999999999999</v>
+        <v>3.3</v>
       </c>
       <c r="U16" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V16" s="15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W16" s="16">
         <f>$S$2*R16+$T$2*S16+$U$2*T16+$V$2*U16-$W$2*V16</f>
@@ -2132,84 +2132,84 @@
         <v>14</v>
       </c>
       <c r="B17" s="18" t="n">
-        <v>3.81</v>
+        <v>3.87</v>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>DeFi rate arbitrage</t>
+          <t>Gaming items</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Borrow-lend spread: USDC on Solana</t>
+          <t>CS2 skins spend-discount (median None% off Steam)</t>
         </is>
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>kamino-lend -&gt; neutral-trade</t>
+          <t>Skinport -&gt; Steam ecosystem</t>
         </is>
       </c>
       <c r="F17" s="20" t="n">
-        <v>8.31</v>
+        <v>22</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>% per year on borrowed notional</t>
+          <t>% discount on Steam spend</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>instant entry/exit</t>
+          <t>instant</t>
         </is>
       </c>
       <c r="I17" s="19" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>unlimited for own spending</t>
         </is>
       </c>
       <c r="J17" s="21" t="n">
-        <v>1066804</v>
+        <v>1000</v>
       </c>
       <c r="K17" s="19" t="inlineStr">
         <is>
-          <t>DefiLlama live rates</t>
+          <t>full 21k-item catalog</t>
         </is>
       </c>
       <c r="L17" s="17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M17" s="17" t="n">
         <v>3</v>
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
+          <t>ONE-WAY: Steam wallet cannot cash out - only worth it for money you'd spend on Steam anyway</t>
         </is>
       </c>
       <c r="O17" s="19" t="inlineStr">
         <is>
-          <t>Borrow USDC at 2.57% on kamino-lend, lend at 10.89% on neutral-trade</t>
+          <t>Buy discounted items on Skinport instead of paying Steam prices</t>
         </is>
       </c>
       <c r="P17" s="22" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="17" t="inlineStr">
         <is>
-          <t>2026-08-16T20:29:43Z</t>
+          <t>2026-08-17T08:42:10Z</t>
         </is>
       </c>
       <c r="R17" s="15" t="n">
-        <v>1.7</v>
+        <v>5.5</v>
       </c>
       <c r="S17" s="15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="T17" s="15" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="U17" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V17" s="15" t="n">
         <v>6</v>
@@ -2224,87 +2224,87 @@
         <v>15</v>
       </c>
       <c r="B18" s="18" t="n">
-        <v>3.8</v>
+        <v>3.84</v>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>Prediction structural</t>
+          <t>DeFi rate arbitrage</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: Highest temperature in Buenos Aires on August</t>
+          <t>Borrow-lend spread: USDC on Solana</t>
         </is>
       </c>
       <c r="E18" s="17" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>kamino-lend -&gt; neutral-trade</t>
         </is>
       </c>
       <c r="F18" s="20" t="n">
-        <v>0.241</v>
+        <v>8.27</v>
       </c>
       <c r="G18" s="19" t="inlineStr">
         <is>
-          <t>% per cycle (riskless)</t>
+          <t>% per year on borrowed notional</t>
         </is>
       </c>
       <c r="H18" s="19" t="inlineStr">
         <is>
-          <t>minutes</t>
+          <t>instant entry/exit</t>
         </is>
       </c>
       <c r="I18" s="19" t="inlineStr">
         <is>
-          <t>5-20 (as books refill)</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="J18" s="21" t="n">
-        <v>40</v>
+        <v>1364122</v>
       </c>
       <c r="K18" s="19" t="inlineStr">
         <is>
-          <t>live CLOB, every outcome book</t>
+          <t>DefiLlama live rates</t>
         </is>
       </c>
       <c r="L18" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M18" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Depth-capped; edge locked at fill; no-fee venue</t>
+          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
         </is>
       </c>
       <c r="O18" s="19" t="inlineStr">
         <is>
-          <t>Buy NO on all 11 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
+          <t>Borrow USDC at 2.29% on kamino-lend, lend at 10.56% on neutral-trade</t>
         </is>
       </c>
       <c r="P18" s="22" t="n">
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="Q18" s="17" t="inlineStr">
         <is>
-          <t>2026-08-17T04:42:19Z</t>
+          <t>2026-08-17T08:42:10Z</t>
         </is>
       </c>
       <c r="R18" s="15" t="n">
-        <v>2.8</v>
+        <v>1.7</v>
       </c>
       <c r="S18" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="T18" s="15" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="U18" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="T18" s="15" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="U18" s="15" t="n">
-        <v>8</v>
-      </c>
       <c r="V18" s="15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="W18" s="16">
         <f>$S$2*R18+$T$2*S18+$U$2*T18+$V$2*U18-$W$2*V18</f>
@@ -2316,7 +2316,7 @@
         <v>16</v>
       </c>
       <c r="B19" s="18" t="n">
-        <v>3.79</v>
+        <v>3.82</v>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: Al Ta'ee Saudi Club vs. Al Qadisiyah Saudi Cl</t>
+          <t>Ladder violation: Will Solana reach $320 by December 31, 2</t>
         </is>
       </c>
       <c r="E19" s="17" t="inlineStr">
@@ -2334,29 +2334,29 @@
         </is>
       </c>
       <c r="F19" s="20" t="n">
-        <v>0.351</v>
+        <v>1.11</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>% per cycle (riskless)</t>
+          <t>% locked at fill</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>minutes</t>
+          <t>instant fill; pays at resolution</t>
         </is>
       </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
-          <t>5-20 (as books refill)</t>
+          <t>when flagged (few/week)</t>
         </is>
       </c>
       <c r="J19" s="21" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K19" s="19" t="inlineStr">
         <is>
-          <t>live CLOB, every outcome book</t>
+          <t>live CLOB depth</t>
         </is>
       </c>
       <c r="L19" s="17" t="n">
@@ -2367,30 +2367,30 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Depth-capped; edge locked at fill; no-fee venue</t>
+          <t>Riskless at fill; capital returns at event resolution; ~$50 size</t>
         </is>
       </c>
       <c r="O19" s="19" t="inlineStr">
         <is>
-          <t>Buy NO on all 3 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
+          <t>Buy YES weaker strike + NO stronger strike for &lt; $1/set; min payout $1, $2 if between strikes</t>
         </is>
       </c>
       <c r="P19" s="22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q19" s="17" t="inlineStr">
         <is>
-          <t>2026-08-17T04:42:19Z</t>
+          <t>2026-08-17T04:43:00Z</t>
         </is>
       </c>
       <c r="R19" s="15" t="n">
-        <v>3.2</v>
+        <v>4.3</v>
       </c>
       <c r="S19" s="15" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="T19" s="15" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="U19" s="15" t="n">
         <v>8</v>
@@ -2472,7 +2472,7 @@
       </c>
       <c r="Q20" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16T20:29:43Z</t>
+          <t>2026-08-17T08:42:10Z</t>
         </is>
       </c>
       <c r="R20" s="15" t="n">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="Q22" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 04:43 UTC</t>
+          <t>2026-08-17 08:42 UTC</t>
         </is>
       </c>
       <c r="R22" s="15" t="n">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="Q23" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 04:43 UTC</t>
+          <t>2026-08-17 08:42 UTC</t>
         </is>
       </c>
       <c r="R23" s="15" t="n">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="Q24" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 04:43 UTC</t>
+          <t>2026-08-17 08:42 UTC</t>
         </is>
       </c>
       <c r="R24" s="15" t="n">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="Q25" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 04:43 UTC</t>
+          <t>2026-08-17 08:42 UTC</t>
         </is>
       </c>
       <c r="R25" s="15" t="n">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="Q26" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 04:43 UTC</t>
+          <t>2026-08-17 08:42 UTC</t>
         </is>
       </c>
       <c r="R26" s="15" t="n">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="Q27" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16T20:29:43Z</t>
+          <t>2026-08-17T08:42:10Z</t>
         </is>
       </c>
       <c r="R27" s="15" t="n">
@@ -3300,7 +3300,7 @@
       </c>
       <c r="Q29" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 04:43 UTC</t>
+          <t>2026-08-17 08:42 UTC</t>
         </is>
       </c>
       <c r="R29" s="15" t="n">
@@ -3604,7 +3604,7 @@
         <v>30</v>
       </c>
       <c r="B33" s="23" t="n">
-        <v>1.58</v>
+        <v>1.52</v>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="F33" s="16" t="n">
-        <v>12.23</v>
+        <v>11.45</v>
       </c>
       <c r="G33" s="24" t="inlineStr">
         <is>
@@ -3668,11 +3668,11 @@
       </c>
       <c r="Q33" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16T20:29:43Z</t>
+          <t>2026-08-17T08:42:10Z</t>
         </is>
       </c>
       <c r="R33" s="15" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="S33" s="15" t="n">
         <v>3</v>
@@ -3714,7 +3714,7 @@
         </is>
       </c>
       <c r="F34" s="16" t="n">
-        <v>6.07</v>
+        <v>6</v>
       </c>
       <c r="G34" s="24" t="inlineStr">
         <is>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="Q34" s="15" t="inlineStr">
         <is>
-          <t>2026-08-16T20:29:43Z</t>
+          <t>2026-08-17T08:42:10Z</t>
         </is>
       </c>
       <c r="R34" s="15" t="n">
@@ -3866,16 +3866,16 @@
         <v>3</v>
       </c>
       <c r="C2" s="29" t="n">
-        <v>1.012</v>
+        <v>1.011</v>
       </c>
       <c r="D2" s="29" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>1.988</v>
+        <v>1.989</v>
       </c>
       <c r="F2" s="29" t="n">
-        <v>0.604</v>
+        <v>0.553</v>
       </c>
       <c r="G2" s="29" t="n">
         <v>5</v>
@@ -3946,29 +3946,29 @@
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>Al Ta'ee Saudi Club vs. Al Qadisiyah Saudi Club</t>
+          <t>Fed Decision in December?</t>
         </is>
       </c>
       <c r="B5" s="29" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C5" s="29" t="n">
-        <v>1.007</v>
+        <v>1.01</v>
       </c>
       <c r="D5" s="29" t="n">
-        <v>0.007</v>
+        <v>0.01</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>1.993</v>
+        <v>3.99</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.351</v>
+        <v>0.251</v>
       </c>
       <c r="G5" s="29" t="n">
-        <v>0</v>
+        <v>827</v>
       </c>
       <c r="H5" s="29" t="n">
-        <v>0</v>
+        <v>8.27</v>
       </c>
       <c r="I5" s="29" t="inlineStr">
         <is>
@@ -3979,29 +3979,29 @@
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>Fed Decision in December?</t>
+          <t>Fed Decision in October?</t>
         </is>
       </c>
       <c r="B6" s="29" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="29" t="n">
-        <v>1.01</v>
+        <v>1.009</v>
       </c>
       <c r="D6" s="29" t="n">
-        <v>0.01</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>3.99</v>
+        <v>3.991</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.251</v>
+        <v>0.226</v>
       </c>
       <c r="G6" s="29" t="n">
-        <v>782</v>
+        <v>100</v>
       </c>
       <c r="H6" s="29" t="n">
-        <v>7.82</v>
+        <v>0.9</v>
       </c>
       <c r="I6" s="29" t="inlineStr">
         <is>
@@ -4012,62 +4012,50 @@
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>Highest temperature in Buenos Aires on August 18?</t>
+          <t xml:space="preserve">Pro Football: NFC West Champion  </t>
         </is>
       </c>
       <c r="B7" s="29" t="n">
-        <v>11</v>
-      </c>
-      <c r="C7" s="29" t="n">
-        <v>1.024</v>
-      </c>
-      <c r="D7" s="29" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="E7" s="29" t="n">
-        <v>9.976000000000001</v>
-      </c>
-      <c r="F7" s="29" t="n">
-        <v>0.241</v>
-      </c>
-      <c r="G7" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="H7" s="29" t="n">
-        <v>0.1</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="29" t="n"/>
+      <c r="F7" s="29" t="n"/>
+      <c r="G7" s="29" t="n"/>
+      <c r="H7" s="29" t="n"/>
       <c r="I7" s="29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>book_unavailable</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t>Fed Decision in October?</t>
+          <t>Anthropic IPO Closing Market Cap</t>
         </is>
       </c>
       <c r="B8" s="29" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C8" s="29" t="n">
-        <v>1.009</v>
+        <v>1.017</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.017</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>3.991</v>
+        <v>8.983000000000001</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.226</v>
+        <v>0.189</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>100</v>
+        <v>19</v>
       </c>
       <c r="H8" s="29" t="n">
-        <v>0.9</v>
+        <v>0.32</v>
       </c>
       <c r="I8" s="29" t="inlineStr">
         <is>
@@ -4078,11 +4066,11 @@
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pro Football: NFC West Champion  </t>
+          <t>Los Angeles Mayoral Election</t>
         </is>
       </c>
       <c r="B9" s="29" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C9" s="29" t="n"/>
       <c r="D9" s="29" t="n"/>
@@ -4099,77 +4087,53 @@
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
         <is>
-          <t>Anthropic IPO Closing Market Cap</t>
+          <t>NBA: 2027 Eastern Conference Champion</t>
         </is>
       </c>
       <c r="B10" s="29" t="n">
-        <v>10</v>
-      </c>
-      <c r="C10" s="29" t="n">
-        <v>1.016</v>
-      </c>
-      <c r="D10" s="29" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="E10" s="29" t="n">
-        <v>8.984</v>
-      </c>
-      <c r="F10" s="29" t="n">
-        <v>0.178</v>
-      </c>
-      <c r="G10" s="29" t="n">
-        <v>40</v>
-      </c>
-      <c r="H10" s="29" t="n">
-        <v>0.64</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="C10" s="29" t="n"/>
+      <c r="D10" s="29" t="n"/>
+      <c r="E10" s="29" t="n"/>
+      <c r="F10" s="29" t="n"/>
+      <c r="G10" s="29" t="n"/>
+      <c r="H10" s="29" t="n"/>
       <c r="I10" s="29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>book_unavailable</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>Highest temperature in Warsaw on August 17?</t>
+          <t>2026 Midterms: House Popular Vote Margin of Victory</t>
         </is>
       </c>
       <c r="B11" s="29" t="n">
-        <v>11</v>
-      </c>
-      <c r="C11" s="29" t="n">
-        <v>1.021</v>
-      </c>
-      <c r="D11" s="29" t="n">
-        <v>0.021</v>
-      </c>
-      <c r="E11" s="29" t="n">
-        <v>9.978999999999999</v>
-      </c>
-      <c r="F11" s="29" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="G11" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" s="29" t="n">
-        <v>0.04</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C11" s="29" t="n"/>
+      <c r="D11" s="29" t="n"/>
+      <c r="E11" s="29" t="n"/>
+      <c r="F11" s="29" t="n"/>
+      <c r="G11" s="29" t="n"/>
+      <c r="H11" s="29" t="n"/>
       <c r="I11" s="29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>book_unavailable</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
-          <t>Los Angeles Mayoral Election</t>
+          <t>Pro Football: 2027 Champion</t>
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="C12" s="29" t="n"/>
       <c r="D12" s="29" t="n"/>
@@ -4186,32 +4150,44 @@
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>NBA: 2027 Eastern Conference Champion</t>
+          <t>How many Fed rate cuts in 2026?</t>
         </is>
       </c>
       <c r="B13" s="29" t="n">
-        <v>18</v>
-      </c>
-      <c r="C13" s="29" t="n"/>
-      <c r="D13" s="29" t="n"/>
-      <c r="E13" s="29" t="n"/>
-      <c r="F13" s="29" t="n"/>
-      <c r="G13" s="29" t="n"/>
-      <c r="H13" s="29" t="n"/>
+        <v>13</v>
+      </c>
+      <c r="C13" s="29" t="n">
+        <v>1.009</v>
+      </c>
+      <c r="D13" s="29" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="E13" s="29" t="n">
+        <v>11.991</v>
+      </c>
+      <c r="F13" s="29" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="G13" s="29" t="n">
+        <v>785.5</v>
+      </c>
+      <c r="H13" s="29" t="n">
+        <v>7.07</v>
+      </c>
       <c r="I13" s="29" t="inlineStr">
         <is>
-          <t>book_unavailable</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>Pro Football: 2027 Champion</t>
+          <t>NBA: 2027 Champion</t>
         </is>
       </c>
       <c r="B14" s="29" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C14" s="29" t="n"/>
       <c r="D14" s="29" t="n"/>
@@ -4228,11 +4204,11 @@
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>LCK 2026 Season Winner</t>
+          <t>BLAST Open Porto 2026: Winner</t>
         </is>
       </c>
       <c r="B15" s="29" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="C15" s="29" t="n"/>
       <c r="D15" s="29" t="n"/>
@@ -5055,7 +5031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5120,106 +5096,106 @@
         <v>772.5441</v>
       </c>
       <c r="C2" s="29" t="n">
-        <v>875</v>
+        <v>895</v>
       </c>
       <c r="D2" s="29" t="n">
-        <v>867</v>
+        <v>861</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>13.26</v>
+        <v>15.85</v>
       </c>
       <c r="F2" s="29" t="n">
-        <v>12.23</v>
+        <v>11.45</v>
       </c>
       <c r="G2" s="29" t="n">
-        <v>-0.91</v>
+        <v>-3.8</v>
       </c>
       <c r="H2" s="29" t="n">
-        <v>149</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="29" t="inlineStr">
         <is>
-          <t>ARS</t>
+          <t>GHS</t>
         </is>
       </c>
       <c r="B3" s="29" t="n">
-        <v>1488.6984</v>
+        <v>10.970191</v>
       </c>
       <c r="C3" s="29" t="n">
-        <v>1582.7</v>
+        <v>11.73</v>
       </c>
       <c r="D3" s="29" t="n">
-        <v>1579</v>
+        <v>11.72</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>6.31</v>
+        <v>6.93</v>
       </c>
       <c r="F3" s="29" t="n">
-        <v>6.07</v>
+        <v>6.83</v>
       </c>
       <c r="G3" s="29" t="n">
-        <v>-0.23</v>
+        <v>-0.09</v>
       </c>
       <c r="H3" s="29" t="n">
-        <v>156</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="29" t="inlineStr">
         <is>
-          <t>BRL</t>
+          <t>ARS</t>
         </is>
       </c>
       <c r="B4" s="29" t="n">
-        <v>5.185311</v>
+        <v>1488.6984</v>
       </c>
       <c r="C4" s="29" t="n">
-        <v>5.73</v>
+        <v>1589</v>
       </c>
       <c r="D4" s="29" t="n">
-        <v>4.92</v>
+        <v>1578.02</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>10.5</v>
+        <v>6.74</v>
       </c>
       <c r="F4" s="29" t="n">
-        <v>-5.12</v>
+        <v>6</v>
       </c>
       <c r="G4" s="29" t="n">
-        <v>-14.14</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="H4" s="29" t="n">
-        <v>64</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>GHS</t>
+          <t>BRL</t>
         </is>
       </c>
       <c r="B5" s="29" t="n">
-        <v>11.186249</v>
+        <v>5.183604</v>
       </c>
       <c r="C5" s="29" t="n">
-        <v>11.75</v>
+        <v>6.25</v>
       </c>
       <c r="D5" s="29" t="n">
-        <v>11.73</v>
+        <v>4.9</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>5.04</v>
+        <v>20.57</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>4.86</v>
+        <v>-5.47</v>
       </c>
       <c r="G5" s="29" t="n">
-        <v>-0.17</v>
+        <v>-21.6</v>
       </c>
       <c r="H5" s="29" t="n">
-        <v>147</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6">
@@ -5229,249 +5205,249 @@
         </is>
       </c>
       <c r="B6" s="29" t="n">
-        <v>9.298643999999999</v>
+        <v>9.284162</v>
       </c>
       <c r="C6" s="29" t="n">
-        <v>9.76</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D6" s="29" t="n">
         <v>9.710000000000001</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>4.96</v>
+        <v>5.56</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>4.42</v>
+        <v>4.59</v>
       </c>
       <c r="G6" s="29" t="n">
-        <v>-0.51</v>
+        <v>-0.92</v>
       </c>
       <c r="H6" s="29" t="n">
-        <v>263</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>UAH</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="B7" s="29" t="n">
-        <v>44.759236</v>
+        <v>95.610406</v>
       </c>
       <c r="C7" s="29" t="n">
-        <v>45.39</v>
+        <v>118</v>
       </c>
       <c r="D7" s="29" t="n">
-        <v>46.17</v>
+        <v>98.52</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>1.41</v>
+        <v>23.42</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>3.15</v>
+        <v>3.04</v>
       </c>
       <c r="G7" s="29" t="n">
-        <v>1.72</v>
+        <v>-16.51</v>
       </c>
       <c r="H7" s="29" t="n">
-        <v>319</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>NGN</t>
         </is>
       </c>
       <c r="B8" s="29" t="n">
-        <v>95.50348099999999</v>
+        <v>1359.199289</v>
       </c>
       <c r="C8" s="29" t="n">
-        <v>118</v>
+        <v>1395.5</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>98.31</v>
+        <v>1392.8</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>23.56</v>
+        <v>2.67</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>2.94</v>
+        <v>2.47</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>-16.69</v>
+        <v>-0.19</v>
       </c>
       <c r="H8" s="29" t="n">
-        <v>52</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>NGN</t>
+          <t>UAH</t>
         </is>
       </c>
       <c r="B9" s="29" t="n">
-        <v>1358.704328</v>
+        <v>44.699683</v>
       </c>
       <c r="C9" s="29" t="n">
-        <v>1393.6</v>
+        <v>45.29</v>
       </c>
       <c r="D9" s="29" t="n">
-        <v>1392.03</v>
+        <v>45.75</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>2.57</v>
+        <v>1.32</v>
       </c>
       <c r="F9" s="29" t="n">
-        <v>2.45</v>
+        <v>2.35</v>
       </c>
       <c r="G9" s="29" t="n">
-        <v>-0.11</v>
+        <v>1.02</v>
       </c>
       <c r="H9" s="29" t="n">
-        <v>250</v>
+        <v>349</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
         <is>
-          <t>LKR</t>
+          <t>PKR</t>
         </is>
       </c>
       <c r="B10" s="29" t="n">
-        <v>333.198729</v>
+        <v>277.654188</v>
       </c>
       <c r="C10" s="29" t="n">
-        <v>367</v>
+        <v>284.4</v>
       </c>
       <c r="D10" s="29" t="n">
-        <v>326.07</v>
+        <v>283.89</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>10.14</v>
+        <v>2.43</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>-2.14</v>
+        <v>2.25</v>
       </c>
       <c r="G10" s="29" t="n">
-        <v>-11.15</v>
+        <v>-0.18</v>
       </c>
       <c r="H10" s="29" t="n">
-        <v>42</v>
+        <v>333</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>EGP</t>
+          <t>TRY</t>
         </is>
       </c>
       <c r="B11" s="29" t="n">
-        <v>50.274761</v>
+        <v>47.884451</v>
       </c>
       <c r="C11" s="29" t="n">
-        <v>50.97</v>
+        <v>49.97</v>
       </c>
       <c r="D11" s="29" t="n">
-        <v>51.31</v>
+        <v>48.91</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>1.38</v>
+        <v>4.36</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>2.06</v>
+        <v>2.14</v>
       </c>
       <c r="G11" s="29" t="n">
-        <v>0.67</v>
+        <v>-2.12</v>
       </c>
       <c r="H11" s="29" t="n">
-        <v>218</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
-          <t>PKR</t>
+          <t>EGP</t>
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>277.780558</v>
+        <v>50.257428</v>
       </c>
       <c r="C12" s="29" t="n">
-        <v>284.12</v>
+        <v>50.94</v>
       </c>
       <c r="D12" s="29" t="n">
-        <v>283.38</v>
+        <v>51.23</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>2.28</v>
+        <v>1.36</v>
       </c>
       <c r="F12" s="29" t="n">
-        <v>2.02</v>
+        <v>1.94</v>
       </c>
       <c r="G12" s="29" t="n">
-        <v>-0.26</v>
+        <v>0.57</v>
       </c>
       <c r="H12" s="29" t="n">
-        <v>231</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>TRY</t>
+          <t>VND</t>
         </is>
       </c>
       <c r="B13" s="29" t="n">
-        <v>47.887954</v>
+        <v>26065.195054</v>
       </c>
       <c r="C13" s="29" t="n">
-        <v>51</v>
+        <v>25800</v>
       </c>
       <c r="D13" s="29" t="n">
-        <v>48.8</v>
+        <v>25796</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>6.5</v>
+        <v>-1.02</v>
       </c>
       <c r="F13" s="29" t="n">
-        <v>1.9</v>
+        <v>-1.03</v>
       </c>
       <c r="G13" s="29" t="n">
-        <v>-4.31</v>
+        <v>-0.02</v>
       </c>
       <c r="H13" s="29" t="n">
-        <v>221</v>
+        <v>400</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>VND</t>
+          <t>LKR</t>
         </is>
       </c>
       <c r="B14" s="29" t="n">
-        <v>26072.465562</v>
+        <v>332.495758</v>
       </c>
       <c r="C14" s="29" t="n">
-        <v>25913</v>
+        <v>367</v>
       </c>
       <c r="D14" s="29" t="n">
-        <v>25843</v>
+        <v>335.54</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>-0.61</v>
+        <v>10.38</v>
       </c>
       <c r="F14" s="29" t="n">
-        <v>-0.88</v>
+        <v>0.92</v>
       </c>
       <c r="G14" s="29" t="n">
-        <v>-0.27</v>
+        <v>-8.57</v>
       </c>
       <c r="H14" s="29" t="n">
-        <v>322</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15">
@@ -5481,81 +5457,81 @@
         </is>
       </c>
       <c r="B15" s="29" t="n">
-        <v>3137.738998</v>
+        <v>3124.110043</v>
       </c>
       <c r="C15" s="29" t="n">
-        <v>3144</v>
+        <v>3149</v>
       </c>
       <c r="D15" s="29" t="n">
-        <v>3110</v>
+        <v>3108.02</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="F15" s="29" t="n">
-        <v>-0.88</v>
+        <v>-0.52</v>
       </c>
       <c r="G15" s="29" t="n">
-        <v>-1.08</v>
+        <v>-1.3</v>
       </c>
       <c r="H15" s="29" t="n">
-        <v>169</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>KES</t>
+          <t>BDT</t>
         </is>
       </c>
       <c r="B16" s="29" t="n">
-        <v>129.213997</v>
+        <v>122.722063</v>
       </c>
       <c r="C16" s="29" t="n">
-        <v>129.15</v>
+        <v>128.94</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>128.56</v>
+        <v>122.19</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>-0.05</v>
+        <v>5.07</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>-0.51</v>
+        <v>-0.43</v>
       </c>
       <c r="G16" s="29" t="n">
-        <v>-0.46</v>
+        <v>-5.23</v>
       </c>
       <c r="H16" s="29" t="n">
-        <v>145</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="29" t="inlineStr">
         <is>
-          <t>IDR</t>
+          <t>KES</t>
         </is>
       </c>
       <c r="B17" s="29" t="n">
-        <v>17822.228665</v>
+        <v>129.238899</v>
       </c>
       <c r="C17" s="29" t="n">
-        <v>17865</v>
+        <v>129</v>
       </c>
       <c r="D17" s="29" t="n">
-        <v>17739</v>
+        <v>128.8</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.24</v>
+        <v>-0.18</v>
       </c>
       <c r="F17" s="29" t="n">
-        <v>-0.47</v>
+        <v>-0.34</v>
       </c>
       <c r="G17" s="29" t="n">
-        <v>-0.71</v>
+        <v>-0.16</v>
       </c>
       <c r="H17" s="29" t="n">
-        <v>163</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18">
@@ -5565,25 +5541,53 @@
         </is>
       </c>
       <c r="B18" s="29" t="n">
-        <v>61.467872</v>
+        <v>61.516375</v>
       </c>
       <c r="C18" s="29" t="n">
-        <v>61.41</v>
+        <v>61.4</v>
       </c>
       <c r="D18" s="29" t="n">
-        <v>61.22</v>
+        <v>61.31</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>-0.09</v>
+        <v>-0.19</v>
       </c>
       <c r="F18" s="29" t="n">
-        <v>-0.4</v>
+        <v>-0.34</v>
       </c>
       <c r="G18" s="29" t="n">
-        <v>-0.31</v>
+        <v>-0.15</v>
       </c>
       <c r="H18" s="29" t="n">
-        <v>203</v>
+        <v>290</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>IDR</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="n">
+        <v>17833.789555</v>
+      </c>
+      <c r="C19" s="29" t="n">
+        <v>17810</v>
+      </c>
+      <c r="D19" s="29" t="n">
+        <v>17775</v>
+      </c>
+      <c r="E19" s="29" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="F19" s="29" t="n">
+        <v>-0.33</v>
+      </c>
+      <c r="G19" s="29" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="H19" s="29" t="n">
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -5678,7 +5682,7 @@
         <v>0.8</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>3354949</v>
+        <v>3322890</v>
       </c>
       <c r="F2" s="29" t="inlineStr">
         <is>
@@ -5686,93 +5690,93 @@
         </is>
       </c>
       <c r="G2" s="29" t="n">
-        <v>21.52</v>
+        <v>20.09</v>
       </c>
       <c r="H2" s="29" t="n">
-        <v>3828261</v>
+        <v>3930955</v>
       </c>
       <c r="I2" s="29" t="n">
-        <v>20.72</v>
+        <v>19.29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="29" t="inlineStr">
         <is>
-          <t>Avalanche</t>
+          <t>Monad</t>
         </is>
       </c>
       <c r="B3" s="29" t="inlineStr">
         <is>
-          <t>SAVAX</t>
+          <t>USDC</t>
         </is>
       </c>
       <c r="C3" s="29" t="inlineStr">
         <is>
-          <t>benqi-lending</t>
+          <t>neverland</t>
         </is>
       </c>
       <c r="D3" s="29" t="n">
-        <v>2.03</v>
+        <v>3.17</v>
       </c>
       <c r="E3" s="29" t="n">
-        <v>61910344</v>
+        <v>1486652</v>
       </c>
       <c r="F3" s="29" t="inlineStr">
         <is>
-          <t>benqi-staked-avax</t>
+          <t>accountable</t>
         </is>
       </c>
       <c r="G3" s="29" t="n">
-        <v>21.02</v>
+        <v>20.13</v>
       </c>
       <c r="H3" s="29" t="n">
-        <v>143805515</v>
+        <v>7497096</v>
       </c>
       <c r="I3" s="29" t="n">
-        <v>19</v>
+        <v>16.96</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="29" t="inlineStr">
         <is>
-          <t>Monad</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>USDC</t>
+          <t>CVXCRV</t>
         </is>
       </c>
       <c r="C4" s="29" t="inlineStr">
         <is>
-          <t>neverland</t>
+          <t>inverse-finance-firm</t>
         </is>
       </c>
       <c r="D4" s="29" t="n">
-        <v>3.12</v>
+        <v>4.07</v>
       </c>
       <c r="E4" s="29" t="n">
-        <v>1517091</v>
+        <v>1728666</v>
       </c>
       <c r="F4" s="29" t="inlineStr">
         <is>
-          <t>accountable</t>
+          <t>convex-finance</t>
         </is>
       </c>
       <c r="G4" s="29" t="n">
-        <v>20.24</v>
+        <v>12.66</v>
       </c>
       <c r="H4" s="29" t="n">
-        <v>7496989</v>
+        <v>39704747</v>
       </c>
       <c r="I4" s="29" t="n">
-        <v>17.12</v>
+        <v>8.59</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>Sui</t>
+          <t>Solana</t>
         </is>
       </c>
       <c r="B5" s="29" t="inlineStr">
@@ -5782,71 +5786,71 @@
       </c>
       <c r="C5" s="29" t="inlineStr">
         <is>
-          <t>scallop-lend</t>
+          <t>kamino-lend</t>
         </is>
       </c>
       <c r="D5" s="29" t="n">
-        <v>3.56</v>
+        <v>2.29</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>1315079</v>
+        <v>1364122</v>
       </c>
       <c r="F5" s="29" t="inlineStr">
         <is>
-          <t>ember-protocol</t>
+          <t>neutral-trade</t>
         </is>
       </c>
       <c r="G5" s="29" t="n">
-        <v>12</v>
+        <v>10.56</v>
       </c>
       <c r="H5" s="29" t="n">
-        <v>9287773</v>
+        <v>3242236</v>
       </c>
       <c r="I5" s="29" t="n">
-        <v>8.44</v>
+        <v>8.27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>CVXCRV</t>
+          <t>WETH</t>
         </is>
       </c>
       <c r="C6" s="29" t="inlineStr">
         <is>
-          <t>inverse-finance-firm</t>
+          <t>compound-v3</t>
         </is>
       </c>
       <c r="D6" s="29" t="n">
-        <v>4.06</v>
+        <v>0</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>1777701</v>
+        <v>5154799</v>
       </c>
       <c r="F6" s="29" t="inlineStr">
         <is>
-          <t>convex-finance</t>
+          <t>fusion-by-ipor</t>
         </is>
       </c>
       <c r="G6" s="29" t="n">
-        <v>12.5</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="H6" s="29" t="n">
-        <v>40645438</v>
+        <v>3400357</v>
       </c>
       <c r="I6" s="29" t="n">
-        <v>8.44</v>
+        <v>8.130000000000001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>Sui</t>
         </is>
       </c>
       <c r="B7" s="29" t="inlineStr">
@@ -5856,65 +5860,65 @@
       </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
-          <t>kamino-lend</t>
+          <t>scallop-lend</t>
         </is>
       </c>
       <c r="D7" s="29" t="n">
-        <v>2.57</v>
+        <v>3.92</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>1066804</v>
+        <v>1318635</v>
       </c>
       <c r="F7" s="29" t="inlineStr">
         <is>
-          <t>neutral-trade</t>
+          <t>ember-protocol</t>
         </is>
       </c>
       <c r="G7" s="29" t="n">
-        <v>10.89</v>
+        <v>12</v>
       </c>
       <c r="H7" s="29" t="n">
-        <v>3240243</v>
+        <v>9287522</v>
       </c>
       <c r="I7" s="29" t="n">
-        <v>8.31</v>
+        <v>8.08</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
-          <t>WETH</t>
+          <t>SUSDAT</t>
         </is>
       </c>
       <c r="C8" s="29" t="inlineStr">
         <is>
-          <t>compound-v3</t>
+          <t>morpho-blue</t>
         </is>
       </c>
       <c r="D8" s="29" t="n">
-        <v>0</v>
+        <v>10.36</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>5115081</v>
+        <v>9807046</v>
       </c>
       <c r="F8" s="29" t="inlineStr">
         <is>
-          <t>fusion-by-ipor</t>
+          <t>saturn</t>
         </is>
       </c>
       <c r="G8" s="29" t="n">
-        <v>8.1</v>
+        <v>18.4</v>
       </c>
       <c r="H8" s="29" t="n">
-        <v>3368926</v>
+        <v>78293653</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>8.1</v>
+        <v>8.039999999999999</v>
       </c>
     </row>
     <row r="9">
@@ -5937,7 +5941,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>1591869</v>
+        <v>1579797</v>
       </c>
       <c r="F9" s="29" t="inlineStr">
         <is>
@@ -5948,7 +5952,7 @@
         <v>7.9</v>
       </c>
       <c r="H9" s="29" t="n">
-        <v>3826818</v>
+        <v>3798743</v>
       </c>
       <c r="I9" s="29" t="n">
         <v>7.9</v>
@@ -5962,7 +5966,7 @@
       </c>
       <c r="B10" s="29" t="inlineStr">
         <is>
-          <t>USD3</t>
+          <t>APYUSD</t>
         </is>
       </c>
       <c r="C10" s="29" t="inlineStr">
@@ -5971,10 +5975,10 @@
         </is>
       </c>
       <c r="D10" s="29" t="n">
-        <v>7.27</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>2763264</v>
+        <v>1446638</v>
       </c>
       <c r="F10" s="29" t="inlineStr">
         <is>
@@ -5982,235 +5986,235 @@
         </is>
       </c>
       <c r="G10" s="29" t="n">
-        <v>14.39</v>
+        <v>17.18</v>
       </c>
       <c r="H10" s="29" t="n">
-        <v>6713644</v>
+        <v>8774256</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>7.12</v>
+        <v>7.89</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>Monad</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B11" s="29" t="inlineStr">
         <is>
-          <t>CBBTC</t>
+          <t>USD3</t>
         </is>
       </c>
       <c r="C11" s="29" t="inlineStr">
         <is>
-          <t>euler-v2</t>
+          <t>morpho-blue</t>
         </is>
       </c>
       <c r="D11" s="29" t="n">
-        <v>0.52</v>
+        <v>7.02</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>3097778</v>
+        <v>2762995</v>
       </c>
       <c r="F11" s="29" t="inlineStr">
         <is>
-          <t>accountable</t>
+          <t>pendle</t>
         </is>
       </c>
       <c r="G11" s="29" t="n">
-        <v>7.16</v>
+        <v>14.4</v>
       </c>
       <c r="H11" s="29" t="n">
-        <v>5419081</v>
+        <v>6709505</v>
       </c>
       <c r="I11" s="29" t="n">
-        <v>6.64</v>
+        <v>7.38</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Monad</t>
         </is>
       </c>
       <c r="B12" s="29" t="inlineStr">
         <is>
-          <t>APYUSD</t>
+          <t>CBBTC</t>
         </is>
       </c>
       <c r="C12" s="29" t="inlineStr">
         <is>
-          <t>morpho-blue</t>
+          <t>euler-v2</t>
         </is>
       </c>
       <c r="D12" s="29" t="n">
-        <v>10.79</v>
+        <v>0.52</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>6204803</v>
+        <v>3116355</v>
       </c>
       <c r="F12" s="29" t="inlineStr">
         <is>
-          <t>pendle</t>
+          <t>accountable</t>
         </is>
       </c>
       <c r="G12" s="29" t="n">
-        <v>17.19</v>
+        <v>7.07</v>
       </c>
       <c r="H12" s="29" t="n">
-        <v>8757533</v>
+        <v>6954114</v>
       </c>
       <c r="I12" s="29" t="n">
-        <v>6.39</v>
+        <v>6.55</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Solana</t>
         </is>
       </c>
       <c r="B13" s="29" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>MSOL</t>
         </is>
       </c>
       <c r="C13" s="29" t="inlineStr">
         <is>
-          <t>liquity-v1</t>
+          <t>kamino-lend</t>
         </is>
       </c>
       <c r="D13" s="29" t="n">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>112287909</v>
+        <v>2482085</v>
       </c>
       <c r="F13" s="29" t="inlineStr">
         <is>
-          <t>vesper</t>
+          <t>marinade-liquid-staking</t>
         </is>
       </c>
       <c r="G13" s="29" t="n">
-        <v>6.84</v>
+        <v>6.32</v>
       </c>
       <c r="H13" s="29" t="n">
-        <v>3483431</v>
+        <v>177725571</v>
       </c>
       <c r="I13" s="29" t="n">
-        <v>6.34</v>
+        <v>6.31</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>Arbitrum</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B14" s="29" t="inlineStr">
         <is>
-          <t>USDT</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C14" s="29" t="inlineStr">
         <is>
-          <t>compound-v3</t>
+          <t>liquity-v1</t>
         </is>
       </c>
       <c r="D14" s="29" t="n">
-        <v>3.02</v>
+        <v>0.5</v>
       </c>
       <c r="E14" s="29" t="n">
-        <v>8879274</v>
+        <v>113297799</v>
       </c>
       <c r="F14" s="29" t="inlineStr">
         <is>
-          <t>zerobase-cedefi</t>
+          <t>vesper</t>
         </is>
       </c>
       <c r="G14" s="29" t="n">
-        <v>9</v>
+        <v>6.72</v>
       </c>
       <c r="H14" s="29" t="n">
-        <v>7629068</v>
+        <v>3511598</v>
       </c>
       <c r="I14" s="29" t="n">
-        <v>5.98</v>
+        <v>6.22</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>Flare</t>
+          <t>Arbitrum</t>
         </is>
       </c>
       <c r="B15" s="29" t="inlineStr">
         <is>
-          <t>SFLR</t>
+          <t>USDT</t>
         </is>
       </c>
       <c r="C15" s="29" t="inlineStr">
         <is>
-          <t>kinetic</t>
+          <t>compound-v3</t>
         </is>
       </c>
       <c r="D15" s="29" t="n">
-        <v>2.28</v>
+        <v>3.02</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>4629461</v>
+        <v>8877763</v>
       </c>
       <c r="F15" s="29" t="inlineStr">
         <is>
-          <t>sceptre-liquid</t>
+          <t>zerobase-cedefi</t>
         </is>
       </c>
       <c r="G15" s="29" t="n">
-        <v>8.08</v>
+        <v>9</v>
       </c>
       <c r="H15" s="29" t="n">
-        <v>14002609</v>
+        <v>7629414</v>
       </c>
       <c r="I15" s="29" t="n">
-        <v>5.8</v>
+        <v>5.98</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Flare</t>
         </is>
       </c>
       <c r="B16" s="29" t="inlineStr">
         <is>
-          <t>SUSDAT</t>
+          <t>SFLR</t>
         </is>
       </c>
       <c r="C16" s="29" t="inlineStr">
         <is>
-          <t>morpho-blue</t>
+          <t>kinetic</t>
         </is>
       </c>
       <c r="D16" s="29" t="n">
-        <v>12.73</v>
+        <v>2.29</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>9811966</v>
+        <v>4437887</v>
       </c>
       <c r="F16" s="29" t="inlineStr">
         <is>
-          <t>saturn</t>
+          <t>sceptre-liquid</t>
         </is>
       </c>
       <c r="G16" s="29" t="n">
-        <v>18.4</v>
+        <v>8.08</v>
       </c>
       <c r="H16" s="29" t="n">
-        <v>78291813</v>
+        <v>14002182</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>5.67</v>
+        <v>5.79</v>
       </c>
     </row>
     <row r="17">
@@ -6230,10 +6234,10 @@
         </is>
       </c>
       <c r="D17" s="29" t="n">
-        <v>3.2</v>
+        <v>3.21</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>16662211</v>
+        <v>16681263</v>
       </c>
       <c r="F17" s="29" t="inlineStr">
         <is>
@@ -6244,10 +6248,10 @@
         <v>8.76</v>
       </c>
       <c r="H17" s="29" t="n">
-        <v>19175036</v>
+        <v>19176431</v>
       </c>
       <c r="I17" s="29" t="n">
-        <v>5.56</v>
+        <v>5.55</v>
       </c>
     </row>
     <row r="18">
@@ -6270,7 +6274,7 @@
         <v>3.48</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>64164146</v>
+        <v>63739102</v>
       </c>
       <c r="F18" s="29" t="inlineStr">
         <is>
@@ -6281,7 +6285,7 @@
         <v>9</v>
       </c>
       <c r="H18" s="29" t="n">
-        <v>14041016</v>
+        <v>14041150</v>
       </c>
       <c r="I18" s="29" t="n">
         <v>5.52</v>
@@ -6295,70 +6299,70 @@
       </c>
       <c r="B19" s="29" t="inlineStr">
         <is>
-          <t>WETH</t>
+          <t>STRUSD</t>
         </is>
       </c>
       <c r="C19" s="29" t="inlineStr">
         <is>
-          <t>compound-v3</t>
+          <t>morpho-blue</t>
         </is>
       </c>
       <c r="D19" s="29" t="n">
-        <v>0</v>
+        <v>6.36</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>117875947</v>
+        <v>2575081</v>
       </c>
       <c r="F19" s="29" t="inlineStr">
         <is>
-          <t>aave-v3</t>
+          <t>pendle</t>
         </is>
       </c>
       <c r="G19" s="29" t="n">
-        <v>5.2</v>
+        <v>11.71</v>
       </c>
       <c r="H19" s="29" t="n">
-        <v>17796206</v>
+        <v>7047753</v>
       </c>
       <c r="I19" s="29" t="n">
-        <v>5.2</v>
+        <v>5.35</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="29" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B20" s="29" t="inlineStr">
         <is>
-          <t>JITOSOL</t>
+          <t>WETH</t>
         </is>
       </c>
       <c r="C20" s="29" t="inlineStr">
         <is>
-          <t>kamino-lend</t>
+          <t>compound-v3</t>
         </is>
       </c>
       <c r="D20" s="29" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>15513202</v>
+        <v>118840010</v>
       </c>
       <c r="F20" s="29" t="inlineStr">
         <is>
-          <t>jito-liquid-staking</t>
+          <t>aave-v3</t>
         </is>
       </c>
       <c r="G20" s="29" t="n">
-        <v>5.12</v>
+        <v>5.19</v>
       </c>
       <c r="H20" s="29" t="n">
-        <v>751506719</v>
+        <v>17950161</v>
       </c>
       <c r="I20" s="29" t="n">
-        <v>5.11</v>
+        <v>5.19</v>
       </c>
     </row>
     <row r="21">
@@ -6369,7 +6373,7 @@
       </c>
       <c r="B21" s="29" t="inlineStr">
         <is>
-          <t>PSOL</t>
+          <t>JITOSOL</t>
         </is>
       </c>
       <c r="C21" s="29" t="inlineStr">
@@ -6378,98 +6382,98 @@
         </is>
       </c>
       <c r="D21" s="29" t="n">
-        <v>1.26</v>
+        <v>0.01</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>6102782</v>
+        <v>15629774</v>
       </c>
       <c r="F21" s="29" t="inlineStr">
         <is>
-          <t>phantom-sol</t>
+          <t>jito-liquid-staking</t>
         </is>
       </c>
       <c r="G21" s="29" t="n">
-        <v>6.29</v>
+        <v>5.09</v>
       </c>
       <c r="H21" s="29" t="n">
-        <v>124009134</v>
+        <v>756783971</v>
       </c>
       <c r="I21" s="29" t="n">
-        <v>5.03</v>
+        <v>5.08</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="29" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Solana</t>
         </is>
       </c>
       <c r="B22" s="29" t="inlineStr">
         <is>
-          <t>REUSD</t>
+          <t>PSOL</t>
         </is>
       </c>
       <c r="C22" s="29" t="inlineStr">
         <is>
-          <t>fluid-lending</t>
+          <t>kamino-lend</t>
         </is>
       </c>
       <c r="D22" s="29" t="n">
-        <v>5.66</v>
+        <v>1.27</v>
       </c>
       <c r="E22" s="29" t="n">
-        <v>3901628</v>
+        <v>6149140</v>
       </c>
       <c r="F22" s="29" t="inlineStr">
         <is>
-          <t>pendle</t>
+          <t>phantom-sol</t>
         </is>
       </c>
       <c r="G22" s="29" t="n">
-        <v>10.42</v>
+        <v>6.3</v>
       </c>
       <c r="H22" s="29" t="n">
-        <v>8583699</v>
+        <v>124875061</v>
       </c>
       <c r="I22" s="29" t="n">
-        <v>4.76</v>
+        <v>5.03</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="29" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B23" s="29" t="inlineStr">
         <is>
-          <t>MSOL</t>
+          <t>REUSD</t>
         </is>
       </c>
       <c r="C23" s="29" t="inlineStr">
         <is>
-          <t>kamino-lend</t>
+          <t>fluid-lending</t>
         </is>
       </c>
       <c r="D23" s="29" t="n">
-        <v>0.01</v>
+        <v>5.68</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>2463543</v>
+        <v>4000680</v>
       </c>
       <c r="F23" s="29" t="inlineStr">
         <is>
-          <t>marinade-liquid-staking</t>
+          <t>pendle</t>
         </is>
       </c>
       <c r="G23" s="29" t="n">
-        <v>4.7</v>
+        <v>10.41</v>
       </c>
       <c r="H23" s="29" t="n">
-        <v>176793661</v>
+        <v>8585141</v>
       </c>
       <c r="I23" s="29" t="n">
-        <v>4.69</v>
+        <v>4.73</v>
       </c>
     </row>
     <row r="24">
@@ -6489,10 +6493,10 @@
         </is>
       </c>
       <c r="D24" s="29" t="n">
-        <v>1.29</v>
+        <v>1.3</v>
       </c>
       <c r="E24" s="29" t="n">
-        <v>38390726</v>
+        <v>38679102</v>
       </c>
       <c r="F24" s="29" t="inlineStr">
         <is>
@@ -6503,21 +6507,21 @@
         <v>5.85</v>
       </c>
       <c r="H24" s="29" t="n">
-        <v>390282152</v>
+        <v>391730152</v>
       </c>
       <c r="I24" s="29" t="n">
-        <v>4.56</v>
+        <v>4.55</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="29" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="B25" s="29" t="inlineStr">
         <is>
-          <t>STRUSD</t>
+          <t>CBETH</t>
         </is>
       </c>
       <c r="C25" s="29" t="inlineStr">
@@ -6526,135 +6530,135 @@
         </is>
       </c>
       <c r="D25" s="29" t="n">
-        <v>6.96</v>
+        <v>4.74</v>
       </c>
       <c r="E25" s="29" t="n">
-        <v>2576835</v>
+        <v>4303544</v>
       </c>
       <c r="F25" s="29" t="inlineStr">
         <is>
-          <t>pendle</t>
+          <t>fusion-by-ipor</t>
         </is>
       </c>
       <c r="G25" s="29" t="n">
-        <v>11.43</v>
+        <v>8.81</v>
       </c>
       <c r="H25" s="29" t="n">
-        <v>7049860</v>
+        <v>4708104</v>
       </c>
       <c r="I25" s="29" t="n">
-        <v>4.47</v>
+        <v>4.07</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="29" t="inlineStr">
         <is>
-          <t>Arbitrum</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="B26" s="29" t="inlineStr">
         <is>
-          <t>SUSDAI</t>
+          <t>USDC</t>
         </is>
       </c>
       <c r="C26" s="29" t="inlineStr">
         <is>
-          <t>fluid-lending</t>
+          <t>aave-v3</t>
         </is>
       </c>
       <c r="D26" s="29" t="n">
-        <v>6.07</v>
+        <v>4.45</v>
       </c>
       <c r="E26" s="29" t="n">
-        <v>7402750</v>
+        <v>19226395</v>
       </c>
       <c r="F26" s="29" t="inlineStr">
         <is>
-          <t>pendle</t>
+          <t>autofinance</t>
         </is>
       </c>
       <c r="G26" s="29" t="n">
-        <v>10.26</v>
+        <v>8.5</v>
       </c>
       <c r="H26" s="29" t="n">
-        <v>11926554</v>
+        <v>4800210</v>
       </c>
       <c r="I26" s="29" t="n">
-        <v>4.19</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="29" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Arbitrum</t>
         </is>
       </c>
       <c r="B27" s="29" t="inlineStr">
         <is>
-          <t>USDC</t>
+          <t>SUSDAI</t>
         </is>
       </c>
       <c r="C27" s="29" t="inlineStr">
         <is>
-          <t>aave-v3</t>
+          <t>fluid-lending</t>
         </is>
       </c>
       <c r="D27" s="29" t="n">
-        <v>4.46</v>
+        <v>6.19</v>
       </c>
       <c r="E27" s="29" t="n">
-        <v>18906738</v>
+        <v>8008577</v>
       </c>
       <c r="F27" s="29" t="inlineStr">
         <is>
-          <t>autofinance</t>
+          <t>pendle</t>
         </is>
       </c>
       <c r="G27" s="29" t="n">
-        <v>8.5</v>
+        <v>10.06</v>
       </c>
       <c r="H27" s="29" t="n">
-        <v>4800210</v>
+        <v>11926638</v>
       </c>
       <c r="I27" s="29" t="n">
-        <v>4.05</v>
+        <v>3.87</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="29" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Plasma</t>
         </is>
       </c>
       <c r="B28" s="29" t="inlineStr">
         <is>
-          <t>CBETH</t>
+          <t>GHO</t>
         </is>
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>morpho-blue</t>
+          <t>aave-v3</t>
         </is>
       </c>
       <c r="D28" s="29" t="n">
-        <v>4.66</v>
+        <v>3.73</v>
       </c>
       <c r="E28" s="29" t="n">
-        <v>10043546</v>
+        <v>5656651</v>
       </c>
       <c r="F28" s="29" t="inlineStr">
         <is>
-          <t>fusion-by-ipor</t>
+          <t>fluid-lending</t>
         </is>
       </c>
       <c r="G28" s="29" t="n">
-        <v>8.67</v>
+        <v>7.31</v>
       </c>
       <c r="H28" s="29" t="n">
-        <v>4668601</v>
+        <v>9566234</v>
       </c>
       <c r="I28" s="29" t="n">
-        <v>4.02</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="29">
@@ -6674,10 +6678,10 @@
         </is>
       </c>
       <c r="D29" s="29" t="n">
-        <v>1.49</v>
+        <v>1.5</v>
       </c>
       <c r="E29" s="29" t="n">
-        <v>6293885</v>
+        <v>6171617</v>
       </c>
       <c r="F29" s="29" t="inlineStr">
         <is>
@@ -6688,7 +6692,7 @@
         <v>4.99</v>
       </c>
       <c r="H29" s="29" t="n">
-        <v>73327136</v>
+        <v>73248911</v>
       </c>
       <c r="I29" s="29" t="n">
         <v>3.49</v>
@@ -6697,38 +6701,38 @@
     <row r="30">
       <c r="A30" s="29" t="inlineStr">
         <is>
-          <t>Plasma</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="B30" s="29" t="inlineStr">
         <is>
-          <t>GHO</t>
+          <t>SIUSD</t>
         </is>
       </c>
       <c r="C30" s="29" t="inlineStr">
         <is>
-          <t>aave-v3</t>
+          <t>morpho-blue</t>
         </is>
       </c>
       <c r="D30" s="29" t="n">
-        <v>3.75</v>
+        <v>2.49</v>
       </c>
       <c r="E30" s="29" t="n">
-        <v>5517773</v>
+        <v>2769351</v>
       </c>
       <c r="F30" s="29" t="inlineStr">
         <is>
-          <t>fluid-lending</t>
+          <t>infinifi</t>
         </is>
       </c>
       <c r="G30" s="29" t="n">
-        <v>7.05</v>
+        <v>5.82</v>
       </c>
       <c r="H30" s="29" t="n">
-        <v>9718471</v>
+        <v>32450339</v>
       </c>
       <c r="I30" s="29" t="n">
-        <v>3.3</v>
+        <v>3.34</v>
       </c>
     </row>
     <row r="31">
@@ -6748,10 +6752,10 @@
         </is>
       </c>
       <c r="D31" s="29" t="n">
-        <v>3.27</v>
+        <v>3.31</v>
       </c>
       <c r="E31" s="29" t="n">
-        <v>14135400</v>
+        <v>14462592</v>
       </c>
       <c r="F31" s="29" t="inlineStr">
         <is>
@@ -6759,10 +6763,10 @@
         </is>
       </c>
       <c r="G31" s="29" t="n">
-        <v>6.54</v>
+        <v>6.58</v>
       </c>
       <c r="H31" s="29" t="n">
-        <v>115384507</v>
+        <v>114546757</v>
       </c>
       <c r="I31" s="29" t="n">
         <v>3.27</v>

</xml_diff>

<commit_message>
Loop refresh 12:41: sweep rotation
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0131Tm9QwYyPuHrkNkGr7Vys
</commit_message>
<xml_diff>
--- a/arb-scanner/data/Arbitrage_Ledger.xlsx
+++ b/arb-scanner/data/Arbitrage_Ledger.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-17 08:42 UTC from six live scanners: 11 crypto exchanges (~9,500 pairs), Polymarket + Kalshi order books,</t>
+          <t>Generated 2026-08-17 12:48 UTC from six live scanners: 11 crypto exchanges (~9,500 pairs), Polymarket + Kalshi order books,</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>2026-08-17 08:42 UTC</t>
+          <t>2026-08-17 12:48 UTC</t>
         </is>
       </c>
       <c r="R4" s="15" t="n">
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="J8" s="13" t="n">
-        <v>3300</v>
+        <v>3372</v>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>2026-08-17T08:41:52Z</t>
+          <t>2026-08-17T12:48:12Z</t>
         </is>
       </c>
       <c r="R8" s="15" t="n">
@@ -1396,7 +1396,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="10" t="n">
-        <v>4.12</v>
+        <v>4.17</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: RC Celta de Vigo vs. CA Osasuna</t>
+          <t>Neg-risk sweep: Orlando City SC vs. Real Salt Lake</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -1432,7 +1432,7 @@
         </is>
       </c>
       <c r="J9" s="13" t="n">
-        <v>116</v>
+        <v>201</v>
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
@@ -1456,11 +1456,11 @@
         </is>
       </c>
       <c r="P9" s="14" t="n">
-        <v>4.6</v>
+        <v>8.1</v>
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>2026-08-17T08:41:52Z</t>
+          <t>2026-08-17T12:48:12Z</t>
         </is>
       </c>
       <c r="R9" s="15" t="n">
@@ -1470,7 +1470,7 @@
         <v>6</v>
       </c>
       <c r="T9" s="15" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="U9" s="15" t="n">
         <v>8</v>
@@ -1488,7 +1488,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="10" t="n">
-        <v>4.02</v>
+        <v>4.12</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: Fed Decision in October?</t>
+          <t>Neg-risk sweep: RC Celta de Vigo vs. CA Osasuna</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -1506,7 +1506,7 @@
         </is>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.226</v>
+        <v>0.503</v>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="J10" s="13" t="n">
-        <v>399</v>
+        <v>116</v>
       </c>
       <c r="K10" s="11" t="inlineStr">
         <is>
@@ -1544,25 +1544,25 @@
       </c>
       <c r="O10" s="11" t="inlineStr">
         <is>
-          <t>Buy NO on all 5 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
+          <t>Buy NO on all 3 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P10" s="14" t="n">
-        <v>7.2</v>
+        <v>4.6</v>
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>2026-08-17T08:41:52Z</t>
+          <t>2026-08-17T12:48:12Z</t>
         </is>
       </c>
       <c r="R10" s="15" t="n">
-        <v>2.8</v>
+        <v>3.5</v>
       </c>
       <c r="S10" s="15" t="n">
         <v>6</v>
       </c>
       <c r="T10" s="15" t="n">
-        <v>3.9</v>
+        <v>3.1</v>
       </c>
       <c r="U10" s="15" t="n">
         <v>8</v>
@@ -1580,7 +1580,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="10" t="n">
-        <v>4.01</v>
+        <v>4.1</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: How many Fed rate cuts in 2026?</t>
+          <t>Neg-risk sweep: Sweden Parliamentary Election: M Vote Share?</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -1598,7 +1598,7 @@
         </is>
       </c>
       <c r="F11" s="12" t="n">
-        <v>0.075</v>
+        <v>0.334</v>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
@@ -1616,7 +1616,7 @@
         </is>
       </c>
       <c r="J11" s="13" t="n">
-        <v>9419</v>
+        <v>248</v>
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
@@ -1636,25 +1636,25 @@
       </c>
       <c r="O11" s="11" t="inlineStr">
         <is>
-          <t>Buy NO on all 13 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
+          <t>Buy NO on all 4 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P11" s="14" t="n">
-        <v>20</v>
+        <v>6.6</v>
       </c>
       <c r="Q11" s="9" t="inlineStr">
         <is>
-          <t>2026-08-17T08:41:52Z</t>
+          <t>2026-08-17T12:48:12Z</t>
         </is>
       </c>
       <c r="R11" s="15" t="n">
-        <v>1.7</v>
+        <v>3.2</v>
       </c>
       <c r="S11" s="15" t="n">
         <v>6</v>
       </c>
       <c r="T11" s="15" t="n">
-        <v>6</v>
+        <v>3.6</v>
       </c>
       <c r="U11" s="15" t="n">
         <v>8</v>
@@ -1672,87 +1672,87 @@
         <v>9</v>
       </c>
       <c r="B12" s="18" t="n">
-        <v>3.93</v>
+        <v>4.02</v>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>DeFi rate arbitrage</t>
+          <t>Prediction structural</t>
         </is>
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Borrow-lend spread: WETH on Base</t>
+          <t>Neg-risk sweep: Fed Decision in October?</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
         <is>
-          <t>compound-v3 -&gt; fusion-by-ipor</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="F12" s="20" t="n">
-        <v>8.130000000000001</v>
+        <v>0.226</v>
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>% per year on borrowed notional</t>
+          <t>% per cycle (riskless)</t>
         </is>
       </c>
       <c r="H12" s="19" t="inlineStr">
         <is>
-          <t>instant entry/exit</t>
+          <t>minutes</t>
         </is>
       </c>
       <c r="I12" s="19" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>5-20 (as books refill)</t>
         </is>
       </c>
       <c r="J12" s="21" t="n">
-        <v>5154799</v>
+        <v>399</v>
       </c>
       <c r="K12" s="19" t="inlineStr">
         <is>
-          <t>DefiLlama live rates</t>
+          <t>live CLOB, every outcome book</t>
         </is>
       </c>
       <c r="L12" s="17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M12" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
+          <t>Depth-capped; edge locked at fill; no-fee venue</t>
         </is>
       </c>
       <c r="O12" s="19" t="inlineStr">
         <is>
-          <t>Borrow WETH at 0% on compound-v3, lend at 8.13% on fusion-by-ipor</t>
+          <t>Buy NO on all 5 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P12" s="22" t="n">
-        <v>1.6</v>
+        <v>7.2</v>
       </c>
       <c r="Q12" s="17" t="inlineStr">
         <is>
-          <t>2026-08-17T08:42:10Z</t>
+          <t>2026-08-17T12:48:12Z</t>
         </is>
       </c>
       <c r="R12" s="15" t="n">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="S12" s="15" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="T12" s="15" t="n">
-        <v>10</v>
+        <v>3.9</v>
       </c>
       <c r="U12" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V12" s="15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W12" s="16">
         <f>$S$2*R12+$T$2*S12+$U$2*T12+$V$2*U12-$W$2*V12</f>
@@ -1764,87 +1764,87 @@
         <v>10</v>
       </c>
       <c r="B13" s="18" t="n">
-        <v>3.93</v>
+        <v>3.98</v>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>DeFi rate arbitrage</t>
+          <t>Prediction structural</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Borrow-lend spread: SUSDAT on Ethereum</t>
+          <t>Neg-risk sweep: Anthropic IPO Closing Market Cap</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
-          <t>morpho-blue -&gt; saturn</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="F13" s="20" t="n">
-        <v>8.039999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>% per year on borrowed notional</t>
+          <t>% per cycle (riskless)</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>instant entry/exit</t>
+          <t>minutes</t>
         </is>
       </c>
       <c r="I13" s="19" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>5-20 (as books refill)</t>
         </is>
       </c>
       <c r="J13" s="21" t="n">
-        <v>9807046</v>
+        <v>359</v>
       </c>
       <c r="K13" s="19" t="inlineStr">
         <is>
-          <t>DefiLlama live rates</t>
+          <t>live CLOB, every outcome book</t>
         </is>
       </c>
       <c r="L13" s="17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M13" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
+          <t>Depth-capped; edge locked at fill; no-fee venue</t>
         </is>
       </c>
       <c r="O13" s="19" t="inlineStr">
         <is>
-          <t>Borrow SUSDAT at 10.36% on morpho-blue, lend at 18.4% on saturn</t>
+          <t>Buy NO on all 10 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
         </is>
       </c>
       <c r="P13" s="22" t="n">
-        <v>1.5</v>
+        <v>5.8</v>
       </c>
       <c r="Q13" s="17" t="inlineStr">
         <is>
-          <t>2026-08-17T08:42:10Z</t>
+          <t>2026-08-17T12:48:12Z</t>
         </is>
       </c>
       <c r="R13" s="15" t="n">
-        <v>1.6</v>
+        <v>2.7</v>
       </c>
       <c r="S13" s="15" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="T13" s="15" t="n">
-        <v>10</v>
+        <v>3.8</v>
       </c>
       <c r="U13" s="15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V13" s="15" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="W13" s="16">
         <f>$S$2*R13+$T$2*S13+$U$2*T13+$V$2*U13-$W$2*V13</f>
@@ -1856,87 +1856,87 @@
         <v>11</v>
       </c>
       <c r="B14" s="18" t="n">
-        <v>3.91</v>
+        <v>3.93</v>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Prediction structural</t>
+          <t>DeFi rate arbitrage</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: Beşiktaş JK vs. FK Kauno Žalgiris</t>
+          <t>Borrow-lend spread: WETH on Base</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>compound-v3 -&gt; fusion-by-ipor</t>
         </is>
       </c>
       <c r="F14" s="20" t="n">
-        <v>0.553</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="G14" s="19" t="inlineStr">
         <is>
-          <t>% per cycle (riskless)</t>
+          <t>% per year on borrowed notional</t>
         </is>
       </c>
       <c r="H14" s="19" t="inlineStr">
         <is>
-          <t>minutes</t>
+          <t>instant entry/exit</t>
         </is>
       </c>
       <c r="I14" s="19" t="inlineStr">
         <is>
-          <t>5-20 (as books refill)</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="J14" s="21" t="n">
+        <v>5154799</v>
+      </c>
+      <c r="K14" s="19" t="inlineStr">
+        <is>
+          <t>DefiLlama live rates</t>
+        </is>
+      </c>
+      <c r="L14" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="19" t="inlineStr">
+        <is>
+          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
+        </is>
+      </c>
+      <c r="O14" s="19" t="inlineStr">
+        <is>
+          <t>Borrow WETH at 0% on compound-v3, lend at 8.13% on fusion-by-ipor</t>
+        </is>
+      </c>
+      <c r="P14" s="22" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="Q14" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-17T08:42:10Z</t>
+        </is>
+      </c>
+      <c r="R14" s="15" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="S14" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="T14" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="K14" s="19" t="inlineStr">
-        <is>
-          <t>live CLOB, every outcome book</t>
-        </is>
-      </c>
-      <c r="L14" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="M14" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="N14" s="19" t="inlineStr">
-        <is>
-          <t>Depth-capped; edge locked at fill; no-fee venue</t>
-        </is>
-      </c>
-      <c r="O14" s="19" t="inlineStr">
-        <is>
-          <t>Buy NO on all 3 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
-        </is>
-      </c>
-      <c r="P14" s="22" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q14" s="17" t="inlineStr">
-        <is>
-          <t>2026-08-17T08:41:52Z</t>
-        </is>
-      </c>
-      <c r="R14" s="15" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="S14" s="15" t="n">
+      <c r="U14" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="T14" s="15" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="U14" s="15" t="n">
-        <v>8</v>
-      </c>
       <c r="V14" s="15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="W14" s="16">
         <f>$S$2*R14+$T$2*S14+$U$2*T14+$V$2*U14-$W$2*V14</f>
@@ -1948,34 +1948,34 @@
         <v>12</v>
       </c>
       <c r="B15" s="18" t="n">
-        <v>3.9</v>
+        <v>3.93</v>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>Rate arbitrage</t>
+          <t>DeFi rate arbitrage</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>EURC on-chain vs Greek deposit</t>
+          <t>Borrow-lend spread: SUSDAT on Ethereum</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
         <is>
-          <t>Aave v3 Ethereum</t>
+          <t>morpho-blue -&gt; saturn</t>
         </is>
       </c>
       <c r="F15" s="20" t="n">
-        <v>2.6</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>% per year net of bank rate</t>
+          <t>% per year on borrowed notional</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>instant</t>
+          <t>instant entry/exit</t>
         </is>
       </c>
       <c r="I15" s="19" t="inlineStr">
@@ -1984,39 +1984,39 @@
         </is>
       </c>
       <c r="J15" s="21" t="n">
-        <v>11000000</v>
+        <v>9807046</v>
       </c>
       <c r="K15" s="19" t="inlineStr">
         <is>
-          <t>DefiLlama: EURC 2.93% APY, $11M TVL</t>
+          <t>DefiLlama live rates</t>
         </is>
       </c>
       <c r="L15" s="17" t="n">
         <v>3</v>
       </c>
       <c r="M15" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Smart-contract + stablecoin issuer risk; beats ESTR slightly</t>
+          <t>Protocol solvency + rate moves + liquidation; obscure lenders = risk premium</t>
         </is>
       </c>
       <c r="O15" s="19" t="inlineStr">
         <is>
-          <t>Hold EURC, supply on Aave</t>
+          <t>Borrow SUSDAT at 10.36% on morpho-blue, lend at 18.4% on saturn</t>
         </is>
       </c>
       <c r="P15" s="22" t="n">
-        <v>0.7</v>
+        <v>1.5</v>
       </c>
       <c r="Q15" s="17" t="inlineStr">
         <is>
-          <t>2026-08-17 08:42 UTC</t>
+          <t>2026-08-17T08:42:10Z</t>
         </is>
       </c>
       <c r="R15" s="15" t="n">
-        <v>0.5</v>
+        <v>1.6</v>
       </c>
       <c r="S15" s="15" t="n">
         <v>9</v>
@@ -2028,7 +2028,7 @@
         <v>6</v>
       </c>
       <c r="V15" s="15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="W15" s="16">
         <f>$S$2*R15+$T$2*S15+$U$2*T15+$V$2*U15-$W$2*V15</f>
@@ -2040,87 +2040,87 @@
         <v>13</v>
       </c>
       <c r="B16" s="18" t="n">
-        <v>3.88</v>
+        <v>3.9</v>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>Prediction structural</t>
+          <t>Rate arbitrage</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>Neg-risk sweep: Anthropic IPO Closing Market Cap</t>
+          <t>EURC on-chain vs Greek deposit</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Aave v3 Ethereum</t>
         </is>
       </c>
       <c r="F16" s="20" t="n">
-        <v>0.189</v>
+        <v>2.6</v>
       </c>
       <c r="G16" s="19" t="inlineStr">
         <is>
-          <t>% per cycle (riskless)</t>
+          <t>% per year net of bank rate</t>
         </is>
       </c>
       <c r="H16" s="19" t="inlineStr">
         <is>
-          <t>minutes</t>
+          <t>instant</t>
         </is>
       </c>
       <c r="I16" s="19" t="inlineStr">
         <is>
-          <t>5-20 (as books refill)</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="J16" s="21" t="n">
-        <v>171</v>
+        <v>11000000</v>
       </c>
       <c r="K16" s="19" t="inlineStr">
         <is>
-          <t>live CLOB, every outcome book</t>
+          <t>DefiLlama: EURC 2.93% APY, $11M TVL</t>
         </is>
       </c>
       <c r="L16" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="M16" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" s="19" t="inlineStr">
+        <is>
+          <t>Smart-contract + stablecoin issuer risk; beats ESTR slightly</t>
+        </is>
+      </c>
+      <c r="O16" s="19" t="inlineStr">
+        <is>
+          <t>Hold EURC, supply on Aave</t>
+        </is>
+      </c>
+      <c r="P16" s="22" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Q16" s="17" t="inlineStr">
+        <is>
+          <t>2026-08-17 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="R16" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S16" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="T16" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="U16" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="V16" s="15" t="n">
         <v>4</v>
-      </c>
-      <c r="M16" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="N16" s="19" t="inlineStr">
-        <is>
-          <t>Depth-capped; edge locked at fill; no-fee venue</t>
-        </is>
-      </c>
-      <c r="O16" s="19" t="inlineStr">
-        <is>
-          <t>Buy NO on all 10 outcomes, convert set to USDC instantly via NegRiskAdapter, repeat</t>
-        </is>
-      </c>
-      <c r="P16" s="22" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="Q16" s="17" t="inlineStr">
-        <is>
-          <t>2026-08-17T08:41:52Z</t>
-        </is>
-      </c>
-      <c r="R16" s="15" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="S16" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="T16" s="15" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="U16" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="V16" s="15" t="n">
-        <v>2</v>
       </c>
       <c r="W16" s="16">
         <f>$S$2*R16+$T$2*S16+$U$2*T16+$V$2*U16-$W$2*V16</f>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="Q22" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 08:42 UTC</t>
+          <t>2026-08-17 12:48 UTC</t>
         </is>
       </c>
       <c r="R22" s="15" t="n">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="Q23" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 08:42 UTC</t>
+          <t>2026-08-17 12:48 UTC</t>
         </is>
       </c>
       <c r="R23" s="15" t="n">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="Q24" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 08:42 UTC</t>
+          <t>2026-08-17 12:48 UTC</t>
         </is>
       </c>
       <c r="R24" s="15" t="n">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="Q25" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 08:42 UTC</t>
+          <t>2026-08-17 12:48 UTC</t>
         </is>
       </c>
       <c r="R25" s="15" t="n">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="Q26" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 08:42 UTC</t>
+          <t>2026-08-17 12:48 UTC</t>
         </is>
       </c>
       <c r="R26" s="15" t="n">
@@ -3300,7 +3300,7 @@
       </c>
       <c r="Q29" s="15" t="inlineStr">
         <is>
-          <t>2026-08-17 08:42 UTC</t>
+          <t>2026-08-17 12:48 UTC</t>
         </is>
       </c>
       <c r="R29" s="15" t="n">
@@ -3859,29 +3859,29 @@
     <row r="2">
       <c r="A2" s="29" t="inlineStr">
         <is>
-          <t>Beşiktaş JK vs. FK Kauno Žalgiris</t>
+          <t>Orlando City SC vs. Real Salt Lake</t>
         </is>
       </c>
       <c r="B2" s="29" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="29" t="n">
-        <v>1.011</v>
+        <v>1.01</v>
       </c>
       <c r="D2" s="29" t="n">
-        <v>0.011</v>
+        <v>0.01</v>
       </c>
       <c r="E2" s="29" t="n">
-        <v>1.989</v>
+        <v>1.99</v>
       </c>
       <c r="F2" s="29" t="n">
-        <v>0.553</v>
+        <v>0.503</v>
       </c>
       <c r="G2" s="29" t="n">
-        <v>5</v>
+        <v>101</v>
       </c>
       <c r="H2" s="29" t="n">
-        <v>0.06</v>
+        <v>1.01</v>
       </c>
       <c r="I2" s="29" t="inlineStr">
         <is>
@@ -3946,11 +3946,11 @@
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
         <is>
-          <t>Fed Decision in December?</t>
+          <t>Sweden Parliamentary Election: M Vote Share?</t>
         </is>
       </c>
       <c r="B5" s="29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5" s="29" t="n">
         <v>1.01</v>
@@ -3959,16 +3959,16 @@
         <v>0.01</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>3.99</v>
+        <v>2.99</v>
       </c>
       <c r="F5" s="29" t="n">
-        <v>0.251</v>
+        <v>0.334</v>
       </c>
       <c r="G5" s="29" t="n">
-        <v>827</v>
+        <v>83</v>
       </c>
       <c r="H5" s="29" t="n">
-        <v>8.27</v>
+        <v>0.83</v>
       </c>
       <c r="I5" s="29" t="inlineStr">
         <is>
@@ -3979,29 +3979,29 @@
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>Fed Decision in October?</t>
+          <t>Fed Decision in December?</t>
         </is>
       </c>
       <c r="B6" s="29" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="29" t="n">
-        <v>1.009</v>
+        <v>1.01</v>
       </c>
       <c r="D6" s="29" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>3.991</v>
+        <v>3.99</v>
       </c>
       <c r="F6" s="29" t="n">
-        <v>0.226</v>
+        <v>0.251</v>
       </c>
       <c r="G6" s="29" t="n">
-        <v>100</v>
+        <v>845.2</v>
       </c>
       <c r="H6" s="29" t="n">
-        <v>0.9</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="I6" s="29" t="inlineStr">
         <is>
@@ -4012,21 +4012,33 @@
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pro Football: NFC West Champion  </t>
+          <t>Fed Decision in October?</t>
         </is>
       </c>
       <c r="B7" s="29" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="29" t="n"/>
-      <c r="D7" s="29" t="n"/>
-      <c r="E7" s="29" t="n"/>
-      <c r="F7" s="29" t="n"/>
-      <c r="G7" s="29" t="n"/>
-      <c r="H7" s="29" t="n"/>
+      <c r="C7" s="29" t="n">
+        <v>1.009</v>
+      </c>
+      <c r="D7" s="29" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>3.991</v>
+      </c>
+      <c r="F7" s="29" t="n">
+        <v>0.226</v>
+      </c>
+      <c r="G7" s="29" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" s="29" t="n">
+        <v>0.9</v>
+      </c>
       <c r="I7" s="29" t="inlineStr">
         <is>
-          <t>book_unavailable</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -4040,22 +4052,22 @@
         <v>10</v>
       </c>
       <c r="C8" s="29" t="n">
-        <v>1.017</v>
+        <v>1.018</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>8.983000000000001</v>
+        <v>8.981999999999999</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.189</v>
+        <v>0.2</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="H8" s="29" t="n">
-        <v>0.32</v>
+        <v>0.72</v>
       </c>
       <c r="I8" s="29" t="inlineStr">
         <is>
@@ -4066,11 +4078,11 @@
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>Los Angeles Mayoral Election</t>
+          <t xml:space="preserve">Pro Football: NFC West Champion  </t>
         </is>
       </c>
       <c r="B9" s="29" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C9" s="29" t="n"/>
       <c r="D9" s="29" t="n"/>
@@ -4087,11 +4099,11 @@
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
         <is>
-          <t>NBA: 2027 Eastern Conference Champion</t>
+          <t>Los Angeles Mayoral Election</t>
         </is>
       </c>
       <c r="B10" s="29" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="C10" s="29" t="n"/>
       <c r="D10" s="29" t="n"/>
@@ -4108,11 +4120,11 @@
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>2026 Midterms: House Popular Vote Margin of Victory</t>
+          <t>NBA: 2027 Eastern Conference Champion</t>
         </is>
       </c>
       <c r="B11" s="29" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C11" s="29" t="n"/>
       <c r="D11" s="29" t="n"/>
@@ -4129,11 +4141,11 @@
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
-          <t>Pro Football: 2027 Champion</t>
+          <t>The International 2026: Winner</t>
         </is>
       </c>
       <c r="B12" s="29" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="C12" s="29" t="n"/>
       <c r="D12" s="29" t="n"/>
@@ -4150,65 +4162,65 @@
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
         <is>
-          <t>How many Fed rate cuts in 2026?</t>
+          <t>Pro Football: 2027 Champion</t>
         </is>
       </c>
       <c r="B13" s="29" t="n">
-        <v>13</v>
-      </c>
-      <c r="C13" s="29" t="n">
-        <v>1.009</v>
-      </c>
-      <c r="D13" s="29" t="n">
-        <v>0.008999999999999999</v>
-      </c>
-      <c r="E13" s="29" t="n">
-        <v>11.991</v>
-      </c>
-      <c r="F13" s="29" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="G13" s="29" t="n">
-        <v>785.5</v>
-      </c>
-      <c r="H13" s="29" t="n">
-        <v>7.07</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="29" t="n"/>
+      <c r="F13" s="29" t="n"/>
+      <c r="G13" s="29" t="n"/>
+      <c r="H13" s="29" t="n"/>
       <c r="I13" s="29" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>book_unavailable</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
         <is>
-          <t>NBA: 2027 Champion</t>
+          <t>How many Fed rate cuts in 2026?</t>
         </is>
       </c>
       <c r="B14" s="29" t="n">
-        <v>36</v>
-      </c>
-      <c r="C14" s="29" t="n"/>
-      <c r="D14" s="29" t="n"/>
-      <c r="E14" s="29" t="n"/>
-      <c r="F14" s="29" t="n"/>
-      <c r="G14" s="29" t="n"/>
-      <c r="H14" s="29" t="n"/>
+        <v>13</v>
+      </c>
+      <c r="C14" s="29" t="n">
+        <v>1.009</v>
+      </c>
+      <c r="D14" s="29" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="E14" s="29" t="n">
+        <v>11.991</v>
+      </c>
+      <c r="F14" s="29" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="G14" s="29" t="n">
+        <v>948.5</v>
+      </c>
+      <c r="H14" s="29" t="n">
+        <v>8.539999999999999</v>
+      </c>
       <c r="I14" s="29" t="inlineStr">
         <is>
-          <t>book_unavailable</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
         <is>
-          <t>BLAST Open Porto 2026: Winner</t>
+          <t>NBA: 2027 Champion</t>
         </is>
       </c>
       <c r="B15" s="29" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="C15" s="29" t="n"/>
       <c r="D15" s="29" t="n"/>

</xml_diff>